<commit_message>
Usar planilla precio final en pedidos
</commit_message>
<xml_diff>
--- a/PLANILLA 43 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 43 LISTA PRECIO FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/861fc5296d07be93/Escritorio/Vtas MHC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="14_{C61B597C-68DF-4D61-B621-05ECCF9D3BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD0F874A-BD57-4C0A-B3D2-8EF776DDD04F}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="14_{263F4A30-9BAB-4950-9099-663040569D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59FEC09B-1C8A-4C10-AF92-8A5303300D98}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="Cálculo Intereses" sheetId="29" r:id="rId6"/>
     <sheet name="Hoja3" sheetId="28" state="hidden" r:id="rId7"/>
     <sheet name="Respaldo" sheetId="24" state="hidden" r:id="rId8"/>
-    <sheet name="BASE DE DATOS OFICIAL" sheetId="16" state="hidden" r:id="rId9"/>
+    <sheet name="BASE DE DATOS OFICIAL" sheetId="16" r:id="rId9"/>
     <sheet name="BD_COMPARATIVA" sheetId="23" state="hidden" r:id="rId10"/>
     <sheet name="TRAYECTORIA" sheetId="19" state="hidden" r:id="rId11"/>
     <sheet name="DESCUENTO COLE 18" sheetId="20" state="hidden" r:id="rId12"/>
@@ -39,12 +39,12 @@
     <definedName name="hist">#REF!</definedName>
     <definedName name="JEAN">'BD jeans Dama'!#REF!</definedName>
     <definedName name="jeandama">'BD jeans Dama'!#REF!</definedName>
-    <definedName name="jeans">'BD jeans Dama'!$A$1:$F$1422</definedName>
-    <definedName name="jeans2" comment="para búsqueda por código, sin pistola">'BD jeans Dama'!$B$1:$I$434</definedName>
+    <definedName name="jeans">'BD jeans Dama'!$A$1:$F$1424</definedName>
+    <definedName name="jeans2" comment="para búsqueda por código, sin pistola">'BD jeans Dama'!$B$1:$I$436</definedName>
     <definedName name="jeanss">'BD jeans Dama'!#REF!</definedName>
-    <definedName name="jeansss">'BD jeans Dama'!$A$1:$F$4062</definedName>
+    <definedName name="jeansss">'BD jeans Dama'!$A$1:$F$4064</definedName>
     <definedName name="jn">'BD jeans Dama'!#REF!</definedName>
-    <definedName name="jnss">'BD jeans Dama'!$A$2:$F$536</definedName>
+    <definedName name="jnss">'BD jeans Dama'!$A$2:$F$538</definedName>
     <definedName name="L">'BASE DE DATOS OFICIAL'!$A$1:$D$126</definedName>
     <definedName name="mahis">#REF!</definedName>
     <definedName name="matof">'BASE DE DATOS OFICIAL'!$A$16:$AF$371</definedName>
@@ -695,7 +695,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6547" uniqueCount="2222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6553" uniqueCount="2226">
   <si>
     <t>TRANSPORTE</t>
   </si>
@@ -7904,6 +7904,18 @@
   </si>
   <si>
     <t>Fecha</t>
+  </si>
+  <si>
+    <t>Jean Cintura Wide Leg, Croop, azul gravillado.</t>
+  </si>
+  <si>
+    <t>Jean Cintura Wide Leg, Croop, azul Bio oscuro</t>
+  </si>
+  <si>
+    <t>Jaime Sasmay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaime Sasmay </t>
   </si>
 </sst>
 </file>
@@ -10161,7 +10173,7 @@
     <xf numFmtId="42" fontId="43" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="67" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="453">
+  <cellXfs count="454">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -11287,7 +11299,126 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="126" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="106" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="106" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="93" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="25" borderId="93" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="9" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="25" borderId="93" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="25" borderId="93" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="25" borderId="93" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="127" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="116" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="117" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="4" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="71" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="74" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -11295,7 +11426,121 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="41" fillId="9" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="41" fillId="9" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="41" fillId="9" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -11351,241 +11596,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="3" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="3" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="41" fillId="9" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="41" fillId="9" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="41" fillId="9" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="9" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="74" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="71" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="126" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="106" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="106" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="93" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="41" fontId="0" fillId="25" borderId="93" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="9" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="25" borderId="93" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="25" borderId="93" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="41" fontId="0" fillId="25" borderId="93" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="127" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="116" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="117" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="4" xfId="9" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -22531,7 +22546,7 @@
                   <a14:compatExt spid="_x0000_s116737"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000001C80100}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000001C80100}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -22600,7 +22615,7 @@
                   <a14:compatExt spid="_x0000_s116738"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000002C80100}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002C80100}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -22674,7 +22689,7 @@
                   <a14:compatExt spid="_x0000_s112641"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000001B80100}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000001B80100}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -22743,7 +22758,7 @@
                   <a14:compatExt spid="_x0000_s112642"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002B80100}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000002B80100}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -22836,7 +22851,6 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1342" displayName="Tabla1342" ref="A3:AC123" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
-  <autoFilter ref="A3:AC123" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="29">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="RUT" dataDxfId="102" totalsRowDxfId="101"/>
     <tableColumn id="29" xr3:uid="{867FBC6B-4F0F-471A-9871-75601A81C66E}" name="RUT2" dataDxfId="100" totalsRowDxfId="99"/>
@@ -23185,173 +23199,173 @@
       <c r="B1" s="317"/>
       <c r="C1" s="106"/>
       <c r="D1" s="108"/>
-      <c r="E1" s="382" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="382"/>
-      <c r="G1" s="382"/>
-      <c r="H1" s="390" t="s">
+      <c r="E1" s="430" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="430"/>
+      <c r="G1" s="430"/>
+      <c r="H1" s="436" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="391"/>
-      <c r="J1" s="391"/>
-      <c r="K1" s="392"/>
-      <c r="L1" s="402" t="str">
+      <c r="I1" s="437"/>
+      <c r="J1" s="437"/>
+      <c r="K1" s="438"/>
+      <c r="L1" s="396" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,3,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M1" s="403"/>
-      <c r="N1" s="403"/>
-      <c r="O1" s="403"/>
-      <c r="P1" s="403"/>
-      <c r="Q1" s="403"/>
-      <c r="R1" s="403"/>
-      <c r="S1" s="403"/>
-      <c r="T1" s="404"/>
+      <c r="M1" s="397"/>
+      <c r="N1" s="397"/>
+      <c r="O1" s="397"/>
+      <c r="P1" s="397"/>
+      <c r="Q1" s="397"/>
+      <c r="R1" s="397"/>
+      <c r="S1" s="397"/>
+      <c r="T1" s="398"/>
     </row>
     <row r="2" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="203"/>
       <c r="B2" s="318"/>
       <c r="C2" s="107"/>
       <c r="D2" s="109"/>
-      <c r="E2" s="383"/>
-      <c r="F2" s="383"/>
-      <c r="G2" s="383"/>
-      <c r="H2" s="387" t="s">
+      <c r="E2" s="431"/>
+      <c r="F2" s="431"/>
+      <c r="G2" s="431"/>
+      <c r="H2" s="385" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="388"/>
-      <c r="J2" s="388"/>
-      <c r="K2" s="389"/>
-      <c r="L2" s="393" t="str">
+      <c r="I2" s="435"/>
+      <c r="J2" s="435"/>
+      <c r="K2" s="386"/>
+      <c r="L2" s="418" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,19,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M2" s="394"/>
-      <c r="N2" s="394"/>
-      <c r="O2" s="394"/>
-      <c r="P2" s="394"/>
-      <c r="Q2" s="394"/>
-      <c r="R2" s="394"/>
-      <c r="S2" s="394"/>
-      <c r="T2" s="395"/>
+      <c r="M2" s="419"/>
+      <c r="N2" s="419"/>
+      <c r="O2" s="419"/>
+      <c r="P2" s="419"/>
+      <c r="Q2" s="419"/>
+      <c r="R2" s="419"/>
+      <c r="S2" s="419"/>
+      <c r="T2" s="420"/>
     </row>
     <row r="3" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="203"/>
       <c r="B3" s="318"/>
       <c r="C3" s="107"/>
       <c r="D3" s="109"/>
-      <c r="E3" s="384" t="e">
+      <c r="E3" s="432" t="e">
         <f>VLOOKUP(L5,'BASE DE DATOS OFICIAL'!A3:AC166,14,0)</f>
         <v>#N/A</v>
       </c>
-      <c r="F3" s="384"/>
-      <c r="G3" s="384"/>
-      <c r="H3" s="387" t="s">
+      <c r="F3" s="432"/>
+      <c r="G3" s="432"/>
+      <c r="H3" s="385" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="388"/>
-      <c r="J3" s="388"/>
-      <c r="K3" s="389"/>
-      <c r="L3" s="393" t="str">
+      <c r="I3" s="435"/>
+      <c r="J3" s="435"/>
+      <c r="K3" s="386"/>
+      <c r="L3" s="418" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,5,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M3" s="394"/>
-      <c r="N3" s="394"/>
-      <c r="O3" s="394"/>
-      <c r="P3" s="394"/>
-      <c r="Q3" s="394"/>
-      <c r="R3" s="394"/>
-      <c r="S3" s="394"/>
-      <c r="T3" s="395"/>
+      <c r="M3" s="419"/>
+      <c r="N3" s="419"/>
+      <c r="O3" s="419"/>
+      <c r="P3" s="419"/>
+      <c r="Q3" s="419"/>
+      <c r="R3" s="419"/>
+      <c r="S3" s="419"/>
+      <c r="T3" s="420"/>
     </row>
     <row r="4" spans="1:22" ht="22.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="203"/>
       <c r="B4" s="318"/>
       <c r="C4" s="107"/>
       <c r="D4" s="109"/>
-      <c r="E4" s="384"/>
-      <c r="F4" s="384"/>
-      <c r="G4" s="384"/>
-      <c r="H4" s="387" t="s">
+      <c r="E4" s="432"/>
+      <c r="F4" s="432"/>
+      <c r="G4" s="432"/>
+      <c r="H4" s="385" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="388"/>
-      <c r="J4" s="388"/>
-      <c r="K4" s="389"/>
-      <c r="L4" s="398" t="str">
+      <c r="I4" s="435"/>
+      <c r="J4" s="435"/>
+      <c r="K4" s="386"/>
+      <c r="L4" s="423" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,20,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M4" s="398"/>
-      <c r="N4" s="398"/>
-      <c r="O4" s="398"/>
-      <c r="P4" s="398"/>
-      <c r="Q4" s="399"/>
-      <c r="R4" s="399"/>
-      <c r="S4" s="398"/>
-      <c r="T4" s="400"/>
+      <c r="M4" s="423"/>
+      <c r="N4" s="423"/>
+      <c r="O4" s="423"/>
+      <c r="P4" s="423"/>
+      <c r="Q4" s="424"/>
+      <c r="R4" s="424"/>
+      <c r="S4" s="423"/>
+      <c r="T4" s="425"/>
     </row>
     <row r="5" spans="1:22" ht="22.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="318"/>
       <c r="C5" s="107"/>
       <c r="D5" s="109"/>
-      <c r="E5" s="385" t="s">
+      <c r="E5" s="433" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="386"/>
-      <c r="G5" s="386"/>
-      <c r="H5" s="363" t="s">
+      <c r="F5" s="434"/>
+      <c r="G5" s="434"/>
+      <c r="H5" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="364"/>
-      <c r="J5" s="364"/>
-      <c r="K5" s="365"/>
-      <c r="L5" s="401"/>
-      <c r="M5" s="401"/>
-      <c r="N5" s="401"/>
-      <c r="O5" s="401"/>
-      <c r="P5" s="401"/>
-      <c r="Q5" s="396" t="s">
+      <c r="I5" s="406"/>
+      <c r="J5" s="406"/>
+      <c r="K5" s="393"/>
+      <c r="L5" s="429"/>
+      <c r="M5" s="429"/>
+      <c r="N5" s="429"/>
+      <c r="O5" s="429"/>
+      <c r="P5" s="429"/>
+      <c r="Q5" s="421" t="s">
         <v>1</v>
       </c>
-      <c r="R5" s="397"/>
-      <c r="S5" s="407"/>
-      <c r="T5" s="408"/>
+      <c r="R5" s="422"/>
+      <c r="S5" s="401"/>
+      <c r="T5" s="402"/>
     </row>
     <row r="6" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="203"/>
       <c r="B6" s="318"/>
       <c r="C6" s="107"/>
       <c r="D6" s="109"/>
-      <c r="E6" s="386"/>
-      <c r="F6" s="386"/>
-      <c r="G6" s="386"/>
-      <c r="H6" s="363" t="s">
+      <c r="E6" s="434"/>
+      <c r="F6" s="434"/>
+      <c r="G6" s="434"/>
+      <c r="H6" s="392" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="364"/>
-      <c r="J6" s="364"/>
-      <c r="K6" s="365"/>
-      <c r="L6" s="379" t="str">
+      <c r="I6" s="406"/>
+      <c r="J6" s="406"/>
+      <c r="K6" s="393"/>
+      <c r="L6" s="426" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,21,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M6" s="380"/>
-      <c r="N6" s="380"/>
-      <c r="O6" s="380"/>
-      <c r="P6" s="381"/>
-      <c r="Q6" s="363" t="s">
+      <c r="M6" s="427"/>
+      <c r="N6" s="427"/>
+      <c r="O6" s="427"/>
+      <c r="P6" s="428"/>
+      <c r="Q6" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="R6" s="365"/>
-      <c r="S6" s="409" t="str">
+      <c r="R6" s="393"/>
+      <c r="S6" s="403" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,4,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="T6" s="406"/>
+      <c r="T6" s="400"/>
     </row>
     <row r="7" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="203"/>
@@ -23360,35 +23374,35 @@
         <v>24</v>
       </c>
       <c r="D7" s="298"/>
-      <c r="E7" s="377" t="str">
+      <c r="E7" s="450" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,17,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="F7" s="377"/>
-      <c r="G7" s="377"/>
-      <c r="H7" s="363" t="s">
+      <c r="F7" s="450"/>
+      <c r="G7" s="450"/>
+      <c r="H7" s="392" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="364"/>
-      <c r="J7" s="364"/>
-      <c r="K7" s="365"/>
-      <c r="L7" s="379" t="str">
+      <c r="I7" s="406"/>
+      <c r="J7" s="406"/>
+      <c r="K7" s="393"/>
+      <c r="L7" s="426" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,6,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M7" s="380"/>
-      <c r="N7" s="380"/>
-      <c r="O7" s="380"/>
-      <c r="P7" s="381"/>
-      <c r="Q7" s="363" t="s">
+      <c r="M7" s="427"/>
+      <c r="N7" s="427"/>
+      <c r="O7" s="427"/>
+      <c r="P7" s="428"/>
+      <c r="Q7" s="392" t="s">
         <v>7</v>
       </c>
-      <c r="R7" s="365"/>
-      <c r="S7" s="409" t="str">
+      <c r="R7" s="393"/>
+      <c r="S7" s="403" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,18,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="T7" s="406"/>
+      <c r="T7" s="400"/>
     </row>
     <row r="8" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="203"/>
@@ -23397,65 +23411,65 @@
         <v>1081</v>
       </c>
       <c r="D8" s="298"/>
-      <c r="E8" s="377"/>
-      <c r="F8" s="377"/>
-      <c r="G8" s="377"/>
-      <c r="H8" s="363" t="s">
+      <c r="E8" s="450"/>
+      <c r="F8" s="450"/>
+      <c r="G8" s="450"/>
+      <c r="H8" s="392" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="364"/>
-      <c r="J8" s="364"/>
-      <c r="K8" s="365"/>
-      <c r="L8" s="374">
+      <c r="I8" s="406"/>
+      <c r="J8" s="406"/>
+      <c r="K8" s="393"/>
+      <c r="L8" s="447">
         <f ca="1">TODAY()</f>
-        <v>46160</v>
-      </c>
-      <c r="M8" s="375"/>
-      <c r="N8" s="375"/>
-      <c r="O8" s="375"/>
-      <c r="P8" s="376"/>
-      <c r="Q8" s="363" t="s">
+        <v>46162</v>
+      </c>
+      <c r="M8" s="448"/>
+      <c r="N8" s="448"/>
+      <c r="O8" s="448"/>
+      <c r="P8" s="449"/>
+      <c r="Q8" s="392" t="s">
         <v>29</v>
       </c>
-      <c r="R8" s="365"/>
-      <c r="S8" s="405" t="str">
+      <c r="R8" s="393"/>
+      <c r="S8" s="399" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,9,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="T8" s="406"/>
+      <c r="T8" s="400"/>
     </row>
     <row r="9" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="203"/>
       <c r="B9" s="318"/>
       <c r="C9" s="297"/>
       <c r="D9" s="298"/>
-      <c r="E9" s="378" t="s">
+      <c r="E9" s="451" t="s">
         <v>1413</v>
       </c>
-      <c r="F9" s="378"/>
-      <c r="G9" s="378"/>
-      <c r="H9" s="412" t="s">
+      <c r="F9" s="451"/>
+      <c r="G9" s="451"/>
+      <c r="H9" s="407" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="413"/>
-      <c r="J9" s="413"/>
-      <c r="K9" s="414"/>
-      <c r="L9" s="368" t="str">
+      <c r="I9" s="408"/>
+      <c r="J9" s="408"/>
+      <c r="K9" s="409"/>
+      <c r="L9" s="441" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,7,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M9" s="369"/>
-      <c r="N9" s="369"/>
-      <c r="O9" s="369"/>
-      <c r="P9" s="370"/>
-      <c r="Q9" s="387" t="s">
+      <c r="M9" s="442"/>
+      <c r="N9" s="442"/>
+      <c r="O9" s="442"/>
+      <c r="P9" s="443"/>
+      <c r="Q9" s="385" t="s">
         <v>1405</v>
       </c>
-      <c r="R9" s="389"/>
-      <c r="S9" s="423" t="s">
+      <c r="R9" s="386"/>
+      <c r="S9" s="390" t="s">
         <v>2179</v>
       </c>
-      <c r="T9" s="424"/>
+      <c r="T9" s="391"/>
     </row>
     <row r="10" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="203"/>
@@ -23464,26 +23478,26 @@
         <v>25</v>
       </c>
       <c r="D10" s="109"/>
-      <c r="E10" s="378"/>
-      <c r="F10" s="378"/>
-      <c r="G10" s="378"/>
-      <c r="H10" s="363" t="s">
+      <c r="E10" s="451"/>
+      <c r="F10" s="451"/>
+      <c r="G10" s="451"/>
+      <c r="H10" s="392" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="364"/>
-      <c r="J10" s="364"/>
-      <c r="K10" s="365"/>
-      <c r="L10" s="420" t="s">
+      <c r="I10" s="406"/>
+      <c r="J10" s="406"/>
+      <c r="K10" s="393"/>
+      <c r="L10" s="415" t="s">
         <v>1763</v>
       </c>
-      <c r="M10" s="421"/>
-      <c r="N10" s="421"/>
-      <c r="O10" s="421"/>
-      <c r="P10" s="422"/>
-      <c r="Q10" s="387"/>
-      <c r="R10" s="389"/>
-      <c r="S10" s="423"/>
-      <c r="T10" s="424"/>
+      <c r="M10" s="416"/>
+      <c r="N10" s="416"/>
+      <c r="O10" s="416"/>
+      <c r="P10" s="417"/>
+      <c r="Q10" s="385"/>
+      <c r="R10" s="386"/>
+      <c r="S10" s="390"/>
+      <c r="T10" s="391"/>
     </row>
     <row r="11" spans="1:22" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="203"/>
@@ -23492,31 +23506,31 @@
         <v>26</v>
       </c>
       <c r="D11" s="294"/>
-      <c r="E11" s="366">
+      <c r="E11" s="439">
         <v>143011</v>
       </c>
-      <c r="F11" s="366"/>
-      <c r="G11" s="366"/>
-      <c r="H11" s="412" t="s">
+      <c r="F11" s="439"/>
+      <c r="G11" s="439"/>
+      <c r="H11" s="407" t="s">
         <v>1406</v>
       </c>
-      <c r="I11" s="413"/>
-      <c r="J11" s="413"/>
-      <c r="K11" s="414"/>
-      <c r="L11" s="419" t="str">
+      <c r="I11" s="408"/>
+      <c r="J11" s="408"/>
+      <c r="K11" s="409"/>
+      <c r="L11" s="414" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,29,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M11" s="419"/>
-      <c r="N11" s="418" t="s">
+      <c r="M11" s="414"/>
+      <c r="N11" s="413" t="s">
         <v>1410</v>
       </c>
-      <c r="O11" s="418"/>
-      <c r="P11" s="418"/>
-      <c r="Q11" s="363" t="s">
+      <c r="O11" s="413"/>
+      <c r="P11" s="413"/>
+      <c r="Q11" s="392" t="s">
         <v>631</v>
       </c>
-      <c r="R11" s="365"/>
+      <c r="R11" s="393"/>
       <c r="S11" s="209"/>
       <c r="T11" s="127"/>
     </row>
@@ -23525,26 +23539,26 @@
       <c r="B12" s="318"/>
       <c r="C12" s="295"/>
       <c r="D12" s="296"/>
-      <c r="E12" s="367"/>
-      <c r="F12" s="367"/>
-      <c r="G12" s="367"/>
-      <c r="H12" s="371" t="s">
+      <c r="E12" s="440"/>
+      <c r="F12" s="440"/>
+      <c r="G12" s="440"/>
+      <c r="H12" s="444" t="s">
         <v>1412</v>
       </c>
-      <c r="I12" s="372"/>
-      <c r="J12" s="372"/>
-      <c r="K12" s="373"/>
-      <c r="L12" s="415" t="s">
+      <c r="I12" s="445"/>
+      <c r="J12" s="445"/>
+      <c r="K12" s="446"/>
+      <c r="L12" s="410" t="s">
         <v>1407</v>
       </c>
-      <c r="M12" s="416"/>
-      <c r="N12" s="416"/>
-      <c r="O12" s="416"/>
-      <c r="P12" s="417"/>
-      <c r="Q12" s="425" t="s">
+      <c r="M12" s="411"/>
+      <c r="N12" s="411"/>
+      <c r="O12" s="411"/>
+      <c r="P12" s="412"/>
+      <c r="Q12" s="394" t="s">
         <v>1408</v>
       </c>
-      <c r="R12" s="426"/>
+      <c r="R12" s="395"/>
       <c r="S12" s="128" t="s">
         <v>1409</v>
       </c>
@@ -23560,25 +23574,25 @@
       <c r="E13" s="300"/>
       <c r="F13" s="300"/>
       <c r="G13" s="300"/>
-      <c r="H13" s="410">
+      <c r="H13" s="404">
         <v>3800</v>
       </c>
-      <c r="I13" s="410"/>
-      <c r="J13" s="410"/>
-      <c r="K13" s="410"/>
-      <c r="L13" s="411" t="str">
+      <c r="I13" s="404"/>
+      <c r="J13" s="404"/>
+      <c r="K13" s="404"/>
+      <c r="L13" s="405" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,24,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="M13" s="411"/>
-      <c r="N13" s="411"/>
-      <c r="O13" s="411"/>
-      <c r="P13" s="411"/>
-      <c r="Q13" s="431" t="str">
+      <c r="M13" s="405"/>
+      <c r="N13" s="405"/>
+      <c r="O13" s="405"/>
+      <c r="P13" s="405"/>
+      <c r="Q13" s="387" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,25,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
-      <c r="R13" s="431"/>
+      <c r="R13" s="387"/>
       <c r="S13" s="121" t="str">
         <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,26,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
@@ -23637,10 +23651,10 @@
       <c r="P14" s="136" t="s">
         <v>23</v>
       </c>
-      <c r="Q14" s="429" t="s">
+      <c r="Q14" s="383" t="s">
         <v>10</v>
       </c>
-      <c r="R14" s="430"/>
+      <c r="R14" s="384"/>
       <c r="S14" s="133" t="s">
         <v>11</v>
       </c>
@@ -23652,17 +23666,20 @@
     </row>
     <row r="15" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="275"/>
-      <c r="B15" s="321"/>
+      <c r="B15" s="321" t="str">
+        <f t="shared" ref="B15:B41" si="0">IF(A15="","",VLOOKUP(A15,jeans,2,FALSE))</f>
+        <v/>
+      </c>
       <c r="C15" s="110" t="e">
-        <f t="shared" ref="C15:C41" si="0">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,3,FALSE),VLOOKUP(B15,jeans2,2,FALSE))</f>
+        <f t="shared" ref="C15:C41" si="1">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,3,FALSE),VLOOKUP(B15,jeans2,2,FALSE))</f>
         <v>#N/A</v>
       </c>
       <c r="D15" s="110" t="e">
-        <f t="shared" ref="D15:D41" si="1">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,4,FALSE),VLOOKUP(B15,jeans2,3,FALSE))</f>
+        <f t="shared" ref="D15:D41" si="2">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,4,FALSE),VLOOKUP(B15,jeans2,3,FALSE))</f>
         <v>#N/A</v>
       </c>
       <c r="E15" s="114" t="e">
-        <f>IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,5,FALSE),VLOOKUP(B15,jeans2,4,FALSE))</f>
+        <f t="shared" ref="E15:E41" si="3">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,5,FALSE),VLOOKUP(B15,jeans2,4,FALSE))</f>
         <v>#N/A</v>
       </c>
       <c r="F15" s="115"/>
@@ -23677,35 +23694,35 @@
       <c r="O15" s="111"/>
       <c r="P15" s="116"/>
       <c r="Q15" s="288">
-        <f t="shared" ref="Q15:Q41" si="2">SUM($F15:$P15)</f>
+        <f t="shared" ref="Q15:Q41" si="4">SUM($F15:$P15)</f>
         <v>0</v>
       </c>
       <c r="R15" s="289"/>
       <c r="S15" s="122" t="e">
-        <f t="shared" ref="S15:S41" si="3">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,6,FALSE),VLOOKUP(B15,jeans2,5,FALSE))</f>
+        <f t="shared" ref="S15:S41" si="5">IF(A15&lt;&gt;"",VLOOKUP(A15,jeans,6,FALSE),VLOOKUP(B15,jeans2,5,FALSE))</f>
         <v>#N/A</v>
       </c>
       <c r="T15" s="113" t="str">
-        <f t="shared" ref="T15:T16" si="4">IFERROR(Q15*S15,"")</f>
+        <f t="shared" ref="T15:T16" si="6">IFERROR(Q15*S15,"")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="212"/>
       <c r="B16" s="321" t="str">
-        <f t="shared" ref="B16:B41" si="5">IF(A16="","",VLOOKUP(A16,jeans,2,FALSE))</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C16" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D16" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D16" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E16" s="114" t="e">
-        <f t="shared" ref="E16:E41" si="6">IF(A16&lt;&gt;"",VLOOKUP(A16,jeans,4,FALSE),VLOOKUP(B16,jeans2,4,FALSE))</f>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F16" s="115"/>
@@ -23720,35 +23737,35 @@
       <c r="O16" s="111"/>
       <c r="P16" s="116"/>
       <c r="Q16" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R16" s="289"/>
       <c r="S16" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T16" s="113" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="275"/>
       <c r="B17" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C17" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D17" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D17" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E17" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F17" s="115"/>
@@ -23763,12 +23780,12 @@
       <c r="O17" s="111"/>
       <c r="P17" s="116"/>
       <c r="Q17" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R17" s="289"/>
       <c r="S17" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T17" s="113" t="str">
@@ -23779,19 +23796,19 @@
     <row r="18" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="212"/>
       <c r="B18" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C18" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D18" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D18" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E18" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F18" s="115"/>
@@ -23806,12 +23823,12 @@
       <c r="O18" s="111"/>
       <c r="P18" s="116"/>
       <c r="Q18" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R18" s="289"/>
       <c r="S18" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T18" s="113" t="str">
@@ -23822,19 +23839,19 @@
     <row r="19" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="212"/>
       <c r="B19" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C19" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D19" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D19" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E19" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F19" s="115"/>
@@ -23849,12 +23866,12 @@
       <c r="O19" s="111"/>
       <c r="P19" s="116"/>
       <c r="Q19" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R19" s="289"/>
       <c r="S19" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T19" s="113" t="str">
@@ -23865,19 +23882,19 @@
     <row r="20" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="212"/>
       <c r="B20" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C20" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D20" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D20" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E20" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F20" s="115"/>
@@ -23892,12 +23909,12 @@
       <c r="O20" s="111"/>
       <c r="P20" s="116"/>
       <c r="Q20" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R20" s="289"/>
       <c r="S20" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T20" s="113" t="str">
@@ -23908,19 +23925,19 @@
     <row r="21" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="212"/>
       <c r="B21" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C21" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D21" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D21" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E21" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F21" s="115"/>
@@ -23935,12 +23952,12 @@
       <c r="O21" s="111"/>
       <c r="P21" s="116"/>
       <c r="Q21" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R21" s="289"/>
       <c r="S21" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T21" s="113" t="str">
@@ -23951,19 +23968,19 @@
     <row r="22" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="212"/>
       <c r="B22" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C22" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D22" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D22" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E22" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F22" s="115"/>
@@ -23978,12 +23995,12 @@
       <c r="O22" s="111"/>
       <c r="P22" s="116"/>
       <c r="Q22" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R22" s="289"/>
       <c r="S22" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T22" s="113" t="str">
@@ -23994,19 +24011,19 @@
     <row r="23" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="212"/>
       <c r="B23" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C23" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D23" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D23" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E23" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F23" s="115"/>
@@ -24021,12 +24038,12 @@
       <c r="O23" s="111"/>
       <c r="P23" s="116"/>
       <c r="Q23" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R23" s="289"/>
       <c r="S23" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T23" s="113" t="str">
@@ -24037,19 +24054,19 @@
     <row r="24" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="212"/>
       <c r="B24" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C24" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D24" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D24" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E24" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F24" s="115"/>
@@ -24064,12 +24081,12 @@
       <c r="O24" s="111"/>
       <c r="P24" s="116"/>
       <c r="Q24" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R24" s="289"/>
       <c r="S24" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T24" s="113" t="str">
@@ -24080,19 +24097,19 @@
     <row r="25" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="212"/>
       <c r="B25" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C25" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D25" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D25" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E25" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F25" s="115"/>
@@ -24107,12 +24124,12 @@
       <c r="O25" s="111"/>
       <c r="P25" s="116"/>
       <c r="Q25" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R25" s="289"/>
       <c r="S25" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T25" s="113" t="str">
@@ -24123,19 +24140,19 @@
     <row r="26" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="212"/>
       <c r="B26" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C26" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D26" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D26" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E26" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F26" s="115"/>
@@ -24150,12 +24167,12 @@
       <c r="O26" s="111"/>
       <c r="P26" s="116"/>
       <c r="Q26" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R26" s="289"/>
       <c r="S26" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T26" s="113" t="str">
@@ -24166,19 +24183,19 @@
     <row r="27" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C27" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D27" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D27" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E27" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F27" s="115"/>
@@ -24193,12 +24210,12 @@
       <c r="O27" s="111"/>
       <c r="P27" s="116"/>
       <c r="Q27" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R27" s="289"/>
       <c r="S27" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T27" s="113" t="str">
@@ -24209,19 +24226,19 @@
     <row r="28" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="212"/>
       <c r="B28" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C28" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D28" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D28" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E28" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F28" s="115"/>
@@ -24236,12 +24253,12 @@
       <c r="O28" s="111"/>
       <c r="P28" s="116"/>
       <c r="Q28" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R28" s="289"/>
       <c r="S28" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T28" s="113" t="str">
@@ -24252,19 +24269,19 @@
     <row r="29" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="212"/>
       <c r="B29" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C29" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D29" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D29" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E29" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F29" s="115"/>
@@ -24279,12 +24296,12 @@
       <c r="O29" s="111"/>
       <c r="P29" s="116"/>
       <c r="Q29" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R29" s="289"/>
       <c r="S29" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T29" s="113" t="str">
@@ -24295,19 +24312,19 @@
     <row r="30" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="212"/>
       <c r="B30" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C30" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D30" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D30" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E30" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F30" s="115"/>
@@ -24322,12 +24339,12 @@
       <c r="O30" s="111"/>
       <c r="P30" s="116"/>
       <c r="Q30" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R30" s="289"/>
       <c r="S30" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T30" s="113" t="str">
@@ -24338,19 +24355,19 @@
     <row r="31" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="212"/>
       <c r="B31" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C31" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D31" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D31" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E31" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F31" s="115"/>
@@ -24365,12 +24382,12 @@
       <c r="O31" s="111"/>
       <c r="P31" s="116"/>
       <c r="Q31" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R31" s="289"/>
       <c r="S31" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T31" s="113" t="str">
@@ -24381,19 +24398,19 @@
     <row r="32" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="212"/>
       <c r="B32" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C32" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D32" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D32" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E32" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F32" s="115"/>
@@ -24408,12 +24425,12 @@
       <c r="O32" s="111"/>
       <c r="P32" s="116"/>
       <c r="Q32" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R32" s="289"/>
       <c r="S32" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T32" s="113" t="str">
@@ -24424,19 +24441,19 @@
     <row r="33" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="212"/>
       <c r="B33" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C33" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D33" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D33" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E33" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F33" s="115"/>
@@ -24451,12 +24468,12 @@
       <c r="O33" s="111"/>
       <c r="P33" s="116"/>
       <c r="Q33" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R33" s="289"/>
       <c r="S33" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T33" s="113" t="str">
@@ -24467,19 +24484,19 @@
     <row r="34" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="212"/>
       <c r="B34" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C34" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D34" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D34" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E34" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F34" s="115"/>
@@ -24494,12 +24511,12 @@
       <c r="O34" s="111"/>
       <c r="P34" s="116"/>
       <c r="Q34" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R34" s="289"/>
       <c r="S34" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T34" s="113" t="str">
@@ -24510,19 +24527,19 @@
     <row r="35" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="212"/>
       <c r="B35" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C35" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D35" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D35" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E35" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F35" s="115"/>
@@ -24537,12 +24554,12 @@
       <c r="O35" s="111"/>
       <c r="P35" s="116"/>
       <c r="Q35" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R35" s="289"/>
       <c r="S35" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T35" s="113" t="str">
@@ -24553,19 +24570,19 @@
     <row r="36" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="212"/>
       <c r="B36" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C36" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D36" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D36" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E36" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F36" s="115"/>
@@ -24580,12 +24597,12 @@
       <c r="O36" s="111"/>
       <c r="P36" s="116"/>
       <c r="Q36" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R36" s="289"/>
       <c r="S36" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T36" s="113" t="str">
@@ -24596,19 +24613,19 @@
     <row r="37" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="212"/>
       <c r="B37" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C37" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D37" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D37" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E37" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F37" s="115"/>
@@ -24623,12 +24640,12 @@
       <c r="O37" s="111"/>
       <c r="P37" s="116"/>
       <c r="Q37" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R37" s="289"/>
       <c r="S37" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T37" s="113" t="str">
@@ -24639,19 +24656,19 @@
     <row r="38" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="212"/>
       <c r="B38" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C38" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D38" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D38" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E38" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F38" s="115"/>
@@ -24666,12 +24683,12 @@
       <c r="O38" s="111"/>
       <c r="P38" s="116"/>
       <c r="Q38" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R38" s="289"/>
       <c r="S38" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T38" s="113" t="str">
@@ -24682,19 +24699,19 @@
     <row r="39" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="212"/>
       <c r="B39" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C39" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D39" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D39" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E39" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F39" s="115"/>
@@ -24709,12 +24726,12 @@
       <c r="O39" s="111"/>
       <c r="P39" s="116"/>
       <c r="Q39" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R39" s="289"/>
       <c r="S39" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T39" s="113" t="str">
@@ -24729,15 +24746,15 @@
         <v/>
       </c>
       <c r="C40" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D40" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D40" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E40" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F40" s="115"/>
@@ -24752,12 +24769,12 @@
       <c r="O40" s="111"/>
       <c r="P40" s="116"/>
       <c r="Q40" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R40" s="289"/>
       <c r="S40" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T40" s="113" t="str">
@@ -24768,19 +24785,19 @@
     <row r="41" spans="1:20" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="213"/>
       <c r="B41" s="321" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C41" s="110" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="D41" s="110" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
+      <c r="D41" s="110" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
       <c r="E41" s="114" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="F41" s="115"/>
@@ -24795,12 +24812,12 @@
       <c r="O41" s="111"/>
       <c r="P41" s="116"/>
       <c r="Q41" s="288">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="R41" s="289"/>
       <c r="S41" s="122" t="e">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
       <c r="T41" s="113" t="str">
@@ -24834,11 +24851,11 @@
       <c r="N42" s="53"/>
       <c r="O42" s="51"/>
       <c r="P42" s="54"/>
-      <c r="Q42" s="432">
+      <c r="Q42" s="388">
         <f t="shared" ref="Q42:Q59" si="13">SUM($F42:$P42)</f>
         <v>0</v>
       </c>
-      <c r="R42" s="433"/>
+      <c r="R42" s="389"/>
       <c r="S42" s="55" t="str">
         <f t="shared" ref="S42:S59" si="14">IF(A42="","",VLOOKUP(A42,jeans,5,FALSE))</f>
         <v/>
@@ -24874,11 +24891,11 @@
       <c r="N43" s="11"/>
       <c r="O43" s="3"/>
       <c r="P43" s="10"/>
-      <c r="Q43" s="427">
+      <c r="Q43" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R43" s="428"/>
+      <c r="R43" s="382"/>
       <c r="S43" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -24914,11 +24931,11 @@
       <c r="N44" s="11"/>
       <c r="O44" s="3"/>
       <c r="P44" s="10"/>
-      <c r="Q44" s="427">
+      <c r="Q44" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R44" s="428"/>
+      <c r="R44" s="382"/>
       <c r="S44" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -24954,11 +24971,11 @@
       <c r="N45" s="11"/>
       <c r="O45" s="3"/>
       <c r="P45" s="10"/>
-      <c r="Q45" s="427">
+      <c r="Q45" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R45" s="428"/>
+      <c r="R45" s="382"/>
       <c r="S45" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -24994,11 +25011,11 @@
       <c r="N46" s="11"/>
       <c r="O46" s="3"/>
       <c r="P46" s="10"/>
-      <c r="Q46" s="427">
+      <c r="Q46" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R46" s="428"/>
+      <c r="R46" s="382"/>
       <c r="S46" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25034,11 +25051,11 @@
       <c r="N47" s="11"/>
       <c r="O47" s="3"/>
       <c r="P47" s="10"/>
-      <c r="Q47" s="427">
+      <c r="Q47" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R47" s="428"/>
+      <c r="R47" s="382"/>
       <c r="S47" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25074,11 +25091,11 @@
       <c r="N48" s="11"/>
       <c r="O48" s="3"/>
       <c r="P48" s="10"/>
-      <c r="Q48" s="427">
+      <c r="Q48" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R48" s="428"/>
+      <c r="R48" s="382"/>
       <c r="S48" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25114,11 +25131,11 @@
       <c r="N49" s="11"/>
       <c r="O49" s="3"/>
       <c r="P49" s="10"/>
-      <c r="Q49" s="427">
+      <c r="Q49" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R49" s="428"/>
+      <c r="R49" s="382"/>
       <c r="S49" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25154,11 +25171,11 @@
       <c r="N50" s="11"/>
       <c r="O50" s="3"/>
       <c r="P50" s="10"/>
-      <c r="Q50" s="427">
+      <c r="Q50" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R50" s="428"/>
+      <c r="R50" s="382"/>
       <c r="S50" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25194,11 +25211,11 @@
       <c r="N51" s="11"/>
       <c r="O51" s="3"/>
       <c r="P51" s="10"/>
-      <c r="Q51" s="427">
+      <c r="Q51" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R51" s="428"/>
+      <c r="R51" s="382"/>
       <c r="S51" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25234,11 +25251,11 @@
       <c r="N52" s="11"/>
       <c r="O52" s="3"/>
       <c r="P52" s="10"/>
-      <c r="Q52" s="427">
+      <c r="Q52" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R52" s="428"/>
+      <c r="R52" s="382"/>
       <c r="S52" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25274,11 +25291,11 @@
       <c r="N53" s="11"/>
       <c r="O53" s="3"/>
       <c r="P53" s="10"/>
-      <c r="Q53" s="427">
+      <c r="Q53" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R53" s="428"/>
+      <c r="R53" s="382"/>
       <c r="S53" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25314,11 +25331,11 @@
       <c r="N54" s="11"/>
       <c r="O54" s="3"/>
       <c r="P54" s="10"/>
-      <c r="Q54" s="427">
+      <c r="Q54" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R54" s="428"/>
+      <c r="R54" s="382"/>
       <c r="S54" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25354,11 +25371,11 @@
       <c r="N55" s="11"/>
       <c r="O55" s="3"/>
       <c r="P55" s="10"/>
-      <c r="Q55" s="427">
+      <c r="Q55" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R55" s="428"/>
+      <c r="R55" s="382"/>
       <c r="S55" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25394,11 +25411,11 @@
       <c r="N56" s="11"/>
       <c r="O56" s="3"/>
       <c r="P56" s="10"/>
-      <c r="Q56" s="427">
+      <c r="Q56" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R56" s="428"/>
+      <c r="R56" s="382"/>
       <c r="S56" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25434,11 +25451,11 @@
       <c r="N57" s="11"/>
       <c r="O57" s="3"/>
       <c r="P57" s="10"/>
-      <c r="Q57" s="427">
+      <c r="Q57" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R57" s="428"/>
+      <c r="R57" s="382"/>
       <c r="S57" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25474,11 +25491,11 @@
       <c r="N58" s="11"/>
       <c r="O58" s="3"/>
       <c r="P58" s="10"/>
-      <c r="Q58" s="427">
+      <c r="Q58" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R58" s="428"/>
+      <c r="R58" s="382"/>
       <c r="S58" s="12" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25514,11 +25531,11 @@
       <c r="N59" s="42"/>
       <c r="O59" s="40"/>
       <c r="P59" s="43"/>
-      <c r="Q59" s="427">
+      <c r="Q59" s="381">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="R59" s="428"/>
+      <c r="R59" s="382"/>
       <c r="S59" s="44" t="str">
         <f t="shared" si="14"/>
         <v/>
@@ -25547,11 +25564,11 @@
       <c r="N60" s="305"/>
       <c r="O60" s="305"/>
       <c r="P60" s="306"/>
-      <c r="Q60" s="434">
+      <c r="Q60" s="379">
         <f>SUM(Q15:Q59)</f>
         <v>0</v>
       </c>
-      <c r="R60" s="435"/>
+      <c r="R60" s="380"/>
       <c r="S60" s="123" t="s">
         <v>18</v>
       </c>
@@ -25802,6 +25819,56 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="66">
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="E11:G12"/>
+    <mergeCell ref="L9:P9"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L8:P8"/>
+    <mergeCell ref="E7:G8"/>
+    <mergeCell ref="E9:G10"/>
+    <mergeCell ref="L7:P7"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="E3:G4"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="L3:T3"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="L4:T4"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="L6:P6"/>
+    <mergeCell ref="L5:P5"/>
+    <mergeCell ref="L1:T1"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="L13:P13"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="L12:P12"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L10:P10"/>
+    <mergeCell ref="L2:T2"/>
+    <mergeCell ref="S9:T10"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="Q55:R55"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q9:R10"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="Q42:R42"/>
+    <mergeCell ref="Q43:R43"/>
     <mergeCell ref="Q60:R60"/>
     <mergeCell ref="Q44:R44"/>
     <mergeCell ref="Q51:R51"/>
@@ -25818,56 +25885,6 @@
     <mergeCell ref="Q56:R56"/>
     <mergeCell ref="Q57:R57"/>
     <mergeCell ref="Q58:R58"/>
-    <mergeCell ref="Q55:R55"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="Q9:R10"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q42:R42"/>
-    <mergeCell ref="Q43:R43"/>
-    <mergeCell ref="S9:T10"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="L1:T1"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="L13:P13"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L12:P12"/>
-    <mergeCell ref="N11:P11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="L10:P10"/>
-    <mergeCell ref="L2:T2"/>
-    <mergeCell ref="L3:T3"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="L4:T4"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="L6:P6"/>
-    <mergeCell ref="L5:P5"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="E3:G4"/>
-    <mergeCell ref="E5:G6"/>
-    <mergeCell ref="H3:K3"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="H4:K4"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H1:K1"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="E11:G12"/>
-    <mergeCell ref="L9:P9"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L8:P8"/>
-    <mergeCell ref="E7:G8"/>
-    <mergeCell ref="E9:G10"/>
-    <mergeCell ref="L7:P7"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A16 A18:A41">
@@ -29387,12 +29404,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="436" t="s">
+      <c r="A1" s="452" t="s">
         <v>1026</v>
       </c>
-      <c r="B1" s="436"/>
-      <c r="C1" s="436"/>
-      <c r="D1" s="436"/>
+      <c r="B1" s="452"/>
+      <c r="C1" s="452"/>
+      <c r="D1" s="452"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D2" s="27"/>
@@ -29539,13 +29556,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="436" t="s">
+      <c r="A2" s="452" t="s">
         <v>1025</v>
       </c>
-      <c r="B2" s="436"/>
-      <c r="C2" s="436"/>
-      <c r="D2" s="436"/>
-      <c r="E2" s="436"/>
+      <c r="B2" s="452"/>
+      <c r="C2" s="452"/>
+      <c r="D2" s="452"/>
+      <c r="E2" s="452"/>
     </row>
     <row r="4" spans="1:5" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B4" s="30" t="s">
@@ -29940,12 +29957,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="436" t="s">
+      <c r="A1" s="452" t="s">
         <v>1026</v>
       </c>
-      <c r="B1" s="436"/>
-      <c r="C1" s="436"/>
-      <c r="D1" s="436"/>
+      <c r="B1" s="452"/>
+      <c r="C1" s="452"/>
+      <c r="D1" s="452"/>
     </row>
     <row r="2" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="26"/>
@@ -32221,7 +32238,7 @@
   <sheetPr codeName="Hoja2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R436"/>
+  <dimension ref="A1:R438"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="239" bestFit="1" customWidth="1"/>
@@ -41788,45 +41805,87 @@
       <c r="G433" s="350"/>
     </row>
     <row r="434" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A434" s="312">
+      <c r="A434" s="292">
+        <v>143800038</v>
+      </c>
+      <c r="B434" s="349">
+        <v>438000</v>
+      </c>
+      <c r="C434" s="329" t="s">
+        <v>2222</v>
+      </c>
+      <c r="D434" s="46" t="s">
+        <v>677</v>
+      </c>
+      <c r="E434" s="46" t="s">
+        <v>2206</v>
+      </c>
+      <c r="F434" s="282">
+        <v>26990</v>
+      </c>
+      <c r="G434" s="350"/>
+    </row>
+    <row r="435" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A435" s="292">
+        <v>143800138</v>
+      </c>
+      <c r="B435" s="349">
+        <v>438001</v>
+      </c>
+      <c r="C435" s="329" t="s">
+        <v>2223</v>
+      </c>
+      <c r="D435" s="46" t="s">
+        <v>677</v>
+      </c>
+      <c r="E435" s="46" t="s">
+        <v>2206</v>
+      </c>
+      <c r="F435" s="282">
+        <v>26990</v>
+      </c>
+      <c r="G435" s="350"/>
+    </row>
+    <row r="436" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A436" s="312">
         <v>143010038</v>
       </c>
-      <c r="B434" s="349">
+      <c r="B436" s="349">
         <v>430100</v>
       </c>
-      <c r="C434" s="329" t="s">
+      <c r="C436" s="329" t="s">
         <v>2127</v>
       </c>
-      <c r="D434" s="46" t="s">
+      <c r="D436" s="46" t="s">
         <v>676</v>
       </c>
-      <c r="E434" s="46" t="s">
+      <c r="E436" s="46" t="s">
         <v>681</v>
       </c>
-      <c r="F434" s="282">
+      <c r="F436" s="282">
         <v>25990</v>
       </c>
-      <c r="G434" s="46" t="s">
+      <c r="G436" s="46" t="s">
         <v>2137</v>
       </c>
-      <c r="H434" s="46" t="s">
+      <c r="H436" s="46" t="s">
         <v>2139</v>
       </c>
     </row>
-    <row r="435" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A435" s="314">
+    <row r="437" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A437" s="314">
         <v>11111111</v>
       </c>
-      <c r="B435" s="316" t="str">
-        <f t="shared" ref="B435" si="0">MID(A435,2,6)</f>
+      <c r="B437" s="316" t="str">
+        <f t="shared" ref="B437" si="0">MID(A437,2,6)</f>
         <v>111111</v>
       </c>
-      <c r="C435" s="14" t="s">
+      <c r="C437" s="14" t="s">
         <v>1000</v>
       </c>
     </row>
-    <row r="436" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A436" s="292"/>
+    <row r="438" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A438" s="292"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H218:K282">
@@ -41844,14 +41903,14 @@
     <cfRule type="duplicateValues" dxfId="33" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A389">
-    <cfRule type="duplicateValues" dxfId="32" priority="558"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="560"/>
     <cfRule type="duplicateValues" dxfId="31" priority="559"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="560"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="558"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A390">
-    <cfRule type="duplicateValues" dxfId="29" priority="561"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="563"/>
     <cfRule type="duplicateValues" dxfId="28" priority="562"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="563"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="561"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A391">
     <cfRule type="duplicateValues" dxfId="26" priority="7"/>
@@ -41889,14 +41948,14 @@
     <cfRule type="duplicateValues" dxfId="6" priority="553"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A346:B361 A363:B363">
-    <cfRule type="duplicateValues" dxfId="5" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="27"/>
     <cfRule type="duplicateValues" dxfId="4" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A362:B362">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.11811023622047245" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="11" orientation="portrait" r:id="rId1"/>
@@ -41914,223 +41973,223 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="437" t="s">
+      <c r="A1" s="363" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="438"/>
-      <c r="C1" s="439" t="s">
+      <c r="B1" s="364"/>
+      <c r="C1" s="365" t="s">
         <v>2213</v>
       </c>
-      <c r="D1" s="440"/>
+      <c r="D1" s="366"/>
     </row>
     <row r="2" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="437" t="s">
+      <c r="A3" s="363" t="s">
         <v>2214</v>
       </c>
-      <c r="B3" s="441">
+      <c r="B3" s="367">
         <v>8000000</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="442"/>
+      <c r="B4" s="368"/>
     </row>
     <row r="5" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="437" t="s">
+      <c r="A5" s="363" t="s">
         <v>2215</v>
       </c>
-      <c r="B5" s="441">
+      <c r="B5" s="367">
         <v>5000000</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="437" t="s">
+      <c r="A6" s="363" t="s">
         <v>2216</v>
       </c>
-      <c r="B6" s="441">
+      <c r="B6" s="367">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="437" t="s">
+      <c r="A7" s="363" t="s">
         <v>2217</v>
       </c>
-      <c r="B7" s="443">
+      <c r="B7" s="369">
         <v>0.02</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="437" t="s">
+      <c r="A8" s="363" t="s">
         <v>2218</v>
       </c>
-      <c r="B8" s="444">
+      <c r="B8" s="370">
         <v>46183</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="437" t="s">
+      <c r="A9" s="363" t="s">
         <v>2219</v>
       </c>
-      <c r="B9" s="445">
+      <c r="B9" s="371">
         <f>(($B$3-$B$5)*$B$7)*$B$6</f>
         <v>360000</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="446" t="s">
+      <c r="A11" s="372" t="s">
         <v>2220</v>
       </c>
-      <c r="B11" s="447" t="s">
+      <c r="B11" s="373" t="s">
         <v>2221</v>
       </c>
-      <c r="C11" s="448" t="s">
+      <c r="C11" s="374" t="s">
         <v>1082</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="449">
+      <c r="A12" s="375">
         <f>($B$6)-($B$6-1)</f>
         <v>1</v>
       </c>
-      <c r="B12" s="450">
+      <c r="B12" s="376">
         <f>+B8</f>
         <v>46183</v>
       </c>
-      <c r="C12" s="451">
-        <f t="shared" ref="C12:C21" si="0">IF(A12&lt;&gt;"-",(($B$3-$B$5)/10+($B$9/$B$6)),"-")</f>
+      <c r="C12" s="377">
+        <f t="shared" ref="C12" si="0">IF(A12&lt;&gt;"-",(($B$3-$B$5)/10+($B$9/$B$6)),"-")</f>
         <v>360000</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="449" t="str">
+      <c r="A13" s="375" t="str">
         <f>IF($B$6=2,"2",IF($B$6&lt;2,"-","2"))</f>
         <v>2</v>
       </c>
-      <c r="B13" s="450">
+      <c r="B13" s="376">
         <f>IF(A13&lt;&gt;"-",B12+30,"-")</f>
         <v>46213</v>
       </c>
-      <c r="C13" s="451">
+      <c r="C13" s="377">
         <f>IF(A13&lt;&gt;"-",(($B$3-$B$5)/10+($B$9/$B$6)),"-")</f>
         <v>360000</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="449" t="str">
+      <c r="A14" s="375" t="str">
         <f>IF($B$6=3,"3",IF($B$6&lt;3,"-","3"))</f>
         <v>3</v>
       </c>
-      <c r="B14" s="450">
+      <c r="B14" s="376">
         <f>IF(A14&lt;&gt;"-",B13+30,"-")</f>
         <v>46243</v>
       </c>
-      <c r="C14" s="451">
+      <c r="C14" s="377">
         <f t="shared" ref="C14:C21" si="1">IF(A14&lt;&gt;"-",(($B$3-$B$5)/10+($B$9/$B$6)),"-")</f>
         <v>360000</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="449" t="str">
+      <c r="A15" s="375" t="str">
         <f>IF($B$6=4,"4",IF($B$6&lt;4,"-","4"))</f>
         <v>4</v>
       </c>
-      <c r="B15" s="450">
+      <c r="B15" s="376">
         <f t="shared" ref="B15:B21" si="2">IF(A15&lt;&gt;"-",B14+30,"-")</f>
         <v>46273</v>
       </c>
-      <c r="C15" s="451">
+      <c r="C15" s="377">
         <f t="shared" si="1"/>
         <v>360000</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="449" t="str">
+      <c r="A16" s="375" t="str">
         <f>IF($B$6=5,"5",IF($B$6&lt;5,"-","5"))</f>
         <v>5</v>
       </c>
-      <c r="B16" s="450">
+      <c r="B16" s="376">
         <f t="shared" si="2"/>
         <v>46303</v>
       </c>
-      <c r="C16" s="451">
+      <c r="C16" s="377">
         <f t="shared" si="1"/>
         <v>360000</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="449" t="str">
+      <c r="A17" s="375" t="str">
         <f>IF($B$6=6,"6",IF($B$6&lt;6,"-","6"))</f>
         <v>6</v>
       </c>
-      <c r="B17" s="450">
+      <c r="B17" s="376">
         <f t="shared" si="2"/>
         <v>46333</v>
       </c>
-      <c r="C17" s="451">
+      <c r="C17" s="377">
         <f t="shared" si="1"/>
         <v>360000</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="449" t="str">
+      <c r="A18" s="375" t="str">
         <f>IF($B$6=7,"7",IF($B$6&lt;7,"-","7"))</f>
         <v>-</v>
       </c>
-      <c r="B18" s="450" t="str">
+      <c r="B18" s="376" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="C18" s="451" t="str">
+      <c r="C18" s="377" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="449" t="str">
+      <c r="A19" s="375" t="str">
         <f>IF($B$6=8,"8",IF($B$6&lt;8,"-","8"))</f>
         <v>-</v>
       </c>
-      <c r="B19" s="450" t="str">
+      <c r="B19" s="376" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="C19" s="451" t="str">
+      <c r="C19" s="377" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="449" t="str">
+      <c r="A20" s="375" t="str">
         <f>IF($B$6=9,"9",IF($B$6&lt;9,"-","9"))</f>
         <v>-</v>
       </c>
-      <c r="B20" s="450" t="str">
+      <c r="B20" s="376" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="C20" s="451" t="str">
+      <c r="C20" s="377" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="449" t="str">
+      <c r="A21" s="375" t="str">
         <f>IF($B$6=10,"10",IF($B$6&lt;10,"-","10"))</f>
         <v>-</v>
       </c>
-      <c r="B21" s="450" t="str">
+      <c r="B21" s="376" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="C21" s="451" t="str">
+      <c r="C21" s="377" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="452"/>
-      <c r="C22" s="442">
+      <c r="A22" s="378"/>
+      <c r="C22" s="368">
         <f>SUM(C12:C21)</f>
         <v>2160000</v>
       </c>
@@ -55105,7 +55164,7 @@
         <v>633</v>
       </c>
       <c r="G5" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H5" s="67"/>
       <c r="I5" s="64"/>
@@ -55261,7 +55320,7 @@
         <v>1238</v>
       </c>
       <c r="G7" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H7" s="67" t="s">
         <v>1178</v>
@@ -55418,7 +55477,7 @@
         <v>1239</v>
       </c>
       <c r="G9" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H9" s="67" t="s">
         <v>1180</v>
@@ -55804,7 +55863,7 @@
         <v>1241</v>
       </c>
       <c r="G14" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H14" s="77" t="s">
         <v>732</v>
@@ -55882,7 +55941,7 @@
         <v>595</v>
       </c>
       <c r="G15" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H15" s="76" t="s">
         <v>596</v>
@@ -56112,7 +56171,7 @@
         <v>1243</v>
       </c>
       <c r="G18" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H18" s="67" t="s">
         <v>1185</v>
@@ -56351,9 +56410,9 @@
         <v>1245</v>
       </c>
       <c r="G21" s="62" t="s">
-        <v>285</v>
-      </c>
-      <c r="H21" s="67" t="s">
+        <v>2224</v>
+      </c>
+      <c r="H21" s="453" t="s">
         <v>1187</v>
       </c>
       <c r="I21" s="64"/>
@@ -56429,9 +56488,9 @@
         <v>1246</v>
       </c>
       <c r="G22" s="62" t="s">
-        <v>285</v>
-      </c>
-      <c r="H22" s="67" t="s">
+        <v>2224</v>
+      </c>
+      <c r="H22" s="453" t="s">
         <v>1188</v>
       </c>
       <c r="I22" s="64"/>
@@ -56584,7 +56643,7 @@
         <v>1248</v>
       </c>
       <c r="G24" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H24" s="67" t="s">
         <v>1190</v>
@@ -56663,7 +56722,7 @@
         <v>1249</v>
       </c>
       <c r="G25" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H25" s="67" t="s">
         <v>1191</v>
@@ -56891,7 +56950,7 @@
         <v>1251</v>
       </c>
       <c r="G28" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H28" s="77" t="s">
         <v>725</v>
@@ -57047,7 +57106,7 @@
         <v>1253</v>
       </c>
       <c r="G30" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H30" s="67" t="s">
         <v>686</v>
@@ -57205,7 +57264,7 @@
         <v>1255</v>
       </c>
       <c r="G32" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H32" s="67" t="s">
         <v>409</v>
@@ -57435,7 +57494,7 @@
         <v>1256</v>
       </c>
       <c r="G35" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H35" s="67" t="s">
         <v>1196</v>
@@ -57903,7 +57962,7 @@
         <v>1261</v>
       </c>
       <c r="G41" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H41" s="67" t="s">
         <v>1201</v>
@@ -58129,7 +58188,7 @@
         <v>1263</v>
       </c>
       <c r="G44" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H44" s="67" t="s">
         <v>1203</v>
@@ -58485,7 +58544,7 @@
         <v>573</v>
       </c>
       <c r="G49" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H49" s="67" t="s">
         <v>692</v>
@@ -58561,7 +58620,7 @@
         <v>534</v>
       </c>
       <c r="G50" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H50" s="67" t="s">
         <v>1204</v>
@@ -58643,7 +58702,7 @@
         <v>1264</v>
       </c>
       <c r="G51" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H51" s="67" t="s">
         <v>1205</v>
@@ -59776,7 +59835,7 @@
         <v>1274</v>
       </c>
       <c r="G66" s="62" t="s">
-        <v>1237</v>
+        <v>2225</v>
       </c>
       <c r="H66" s="67" t="s">
         <v>613</v>
@@ -59998,7 +60057,7 @@
         <v>1276</v>
       </c>
       <c r="G69" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H69" s="77" t="s">
         <v>1216</v>
@@ -60376,7 +60435,7 @@
         <v>1279</v>
       </c>
       <c r="G74" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H74" s="67" t="s">
         <v>1219</v>
@@ -61341,7 +61400,7 @@
         <v>581</v>
       </c>
       <c r="G87" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H87" s="67" t="s">
         <v>582</v>
@@ -61635,7 +61694,7 @@
         <v>1285</v>
       </c>
       <c r="G91" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H91" s="67"/>
       <c r="I91" s="64"/>
@@ -61790,7 +61849,7 @@
         <v>996407930</v>
       </c>
       <c r="G93" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H93" s="76" t="s">
         <v>690</v>
@@ -61866,7 +61925,7 @@
         <v>1287</v>
       </c>
       <c r="G94" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H94" s="67" t="s">
         <v>1225</v>
@@ -62023,7 +62082,7 @@
         <v>1289</v>
       </c>
       <c r="G96" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H96" s="67" t="s">
         <v>1227</v>
@@ -62102,7 +62161,7 @@
         <v>206</v>
       </c>
       <c r="G97" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H97" s="67" t="s">
         <v>684</v>
@@ -62903,7 +62962,7 @@
         <v>1294</v>
       </c>
       <c r="G107" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H107" s="67" t="s">
         <v>703</v>
@@ -63039,7 +63098,7 @@
         <v>1295</v>
       </c>
       <c r="G109" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H109" s="67" t="s">
         <v>1229</v>
@@ -63836,7 +63895,7 @@
         <v>1300</v>
       </c>
       <c r="G119" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H119" s="67" t="s">
         <v>1232</v>
@@ -64256,7 +64315,7 @@
         <v>700</v>
       </c>
       <c r="G125" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H125" s="67" t="s">
         <v>701</v>
@@ -64323,7 +64382,7 @@
         <v>707</v>
       </c>
       <c r="G126" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H126" s="67" t="s">
         <v>708</v>
@@ -64393,7 +64452,7 @@
         <v>672411298</v>
       </c>
       <c r="G127" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H127" s="67" t="s">
         <v>714</v>
@@ -64466,7 +64525,7 @@
         <v>652671443</v>
       </c>
       <c r="G128" s="62" t="s">
-        <v>632</v>
+        <v>2224</v>
       </c>
       <c r="H128" s="67" t="s">
         <v>719</v>
@@ -64533,7 +64592,7 @@
         <v>953278601</v>
       </c>
       <c r="G129" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H129" s="67" t="s">
         <v>1234</v>
@@ -64597,7 +64656,7 @@
         <v>512751119</v>
       </c>
       <c r="G130" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H130" s="67" t="s">
         <v>734</v>
@@ -64661,7 +64720,7 @@
         <v>958508878</v>
       </c>
       <c r="G131" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H131" s="67" t="s">
         <v>739</v>
@@ -64733,7 +64792,7 @@
         <v>942213276</v>
       </c>
       <c r="G132" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H132" s="67" t="s">
         <v>744</v>
@@ -64797,7 +64856,7 @@
         <v>1303</v>
       </c>
       <c r="G133" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H133" s="67" t="s">
         <v>1235</v>
@@ -64867,7 +64926,7 @@
         <v>927</v>
       </c>
       <c r="G134" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H134" s="67" t="s">
         <v>752</v>
@@ -64931,7 +64990,7 @@
         <v>981379473</v>
       </c>
       <c r="G135" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H135" s="67" t="s">
         <v>755</v>
@@ -65000,7 +65059,7 @@
         <v>761</v>
       </c>
       <c r="G136" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H136" s="67" t="s">
         <v>1236</v>
@@ -65069,7 +65128,7 @@
         <v>953509920</v>
       </c>
       <c r="G137" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H137" s="67" t="s">
         <v>766</v>
@@ -65134,7 +65193,7 @@
         <v>957891348</v>
       </c>
       <c r="G138" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H138" s="67" t="s">
         <v>770</v>
@@ -65200,7 +65259,7 @@
         <v>975857893</v>
       </c>
       <c r="G139" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H139" s="67" t="s">
         <v>771</v>
@@ -65267,7 +65326,7 @@
         <v>941121845</v>
       </c>
       <c r="G140" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H140" s="67" t="s">
         <v>774</v>
@@ -66354,7 +66413,7 @@
         <v>966752904</v>
       </c>
       <c r="G156" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H156" s="67" t="s">
         <v>582</v>
@@ -66744,7 +66803,7 @@
         <v>972</v>
       </c>
       <c r="G162" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H162" s="67" t="s">
         <v>974</v>
@@ -66806,7 +66865,7 @@
         <v>993366440</v>
       </c>
       <c r="G163" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H163" s="67" t="s">
         <v>978</v>
@@ -66867,7 +66926,7 @@
         <v>953484368</v>
       </c>
       <c r="G164" s="62" t="s">
-        <v>285</v>
+        <v>2224</v>
       </c>
       <c r="H164" s="67" t="s">
         <v>982</v>
@@ -67104,17 +67163,19 @@
     <hyperlink ref="H160" r:id="rId66" xr:uid="{00000000-0004-0000-0200-000041000000}"/>
     <hyperlink ref="H165" r:id="rId67" xr:uid="{00000000-0004-0000-0200-000042000000}"/>
     <hyperlink ref="H166" r:id="rId68" xr:uid="{00000000-0004-0000-0200-000043000000}"/>
+    <hyperlink ref="H22" r:id="rId69" xr:uid="{5FAE5429-A3FA-488F-BB1F-046B7A54FF37}"/>
+    <hyperlink ref="H21" r:id="rId70" xr:uid="{4C2ADD26-02E1-4679-88FB-18E0C221F9EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="83" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId69"/>
-  <drawing r:id="rId70"/>
-  <legacyDrawing r:id="rId71"/>
+  <pageSetup paperSize="9" scale="83" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId71"/>
+  <drawing r:id="rId72"/>
+  <legacyDrawing r:id="rId73"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="112641" r:id="rId72" name="Button 1">
+            <control shapeId="112641" r:id="rId74" name="Button 1">
               <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!volver">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
@@ -67136,7 +67197,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="112642" r:id="rId73" name="Button 2">
+            <control shapeId="112642" r:id="rId75" name="Button 2">
               <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!Botón2_Haga_clic_en">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
@@ -67160,7 +67221,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <tableParts count="1">
-    <tablePart r:id="rId74"/>
+    <tablePart r:id="rId76"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: reconstruir PLANILLA 43 preservando XML original (sin reescritura ET)
- Usa manipulación de texto puro para insertar filas y shared strings
- Preserva todos los namespace declarations originales de Excel
- 558 artículos Cole 44 en filas 439-996, jeans2 hasta $I$996
- Sin inlineStr, sin namespace mangling → abre sin error

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLANILLA 43 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 43 LISTA PRECIO FINAL.xlsx
@@ -32723,12 +32723,12 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Hoja2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R438"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="239" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" style="315" bestFit="1" customWidth="1"/>
@@ -32745,7 +32745,7 @@
     <col min="17" max="16384" width="11.44140625" style="46"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="138" customFormat="1" ht="21.6" customHeight="1" ns3:dyDescent="0.3">
+    <row r="1" spans="1:6" s="138" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="240" t="s">
         <v>8</v>
       </c>
@@ -32765,7 +32765,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="241">
         <v>3801</v>
       </c>
@@ -32785,7 +32785,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="241">
         <v>3802</v>
       </c>
@@ -32805,7 +32805,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="241">
         <v>3818</v>
       </c>
@@ -32825,7 +32825,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="241" t="s">
         <v>1037</v>
       </c>
@@ -32845,7 +32845,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="241" t="s">
         <v>1038</v>
       </c>
@@ -32865,7 +32865,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="241">
         <v>3826</v>
       </c>
@@ -32885,7 +32885,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="241" t="s">
         <v>1053</v>
       </c>
@@ -32905,7 +32905,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="241">
         <v>3834</v>
       </c>
@@ -32925,7 +32925,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="242">
         <v>3837</v>
       </c>
@@ -32945,7 +32945,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="242">
         <v>3840</v>
       </c>
@@ -32965,7 +32965,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="241" t="s">
         <v>1039</v>
       </c>
@@ -32985,7 +32985,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="241" t="s">
         <v>1040</v>
       </c>
@@ -33005,7 +33005,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="241" t="s">
         <v>1041</v>
       </c>
@@ -33025,7 +33025,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="241" t="s">
         <v>1042</v>
       </c>
@@ -33045,7 +33045,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="241" t="s">
         <v>1043</v>
       </c>
@@ -33065,7 +33065,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="241">
         <v>3849</v>
       </c>
@@ -33085,7 +33085,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="241" t="s">
         <v>1044</v>
       </c>
@@ -33105,7 +33105,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="241">
         <v>3851</v>
       </c>
@@ -33125,7 +33125,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="241">
         <v>3857</v>
       </c>
@@ -33145,7 +33145,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="241">
         <v>3858</v>
       </c>
@@ -33165,7 +33165,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="241">
         <v>3859</v>
       </c>
@@ -33183,7 +33183,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="241">
         <v>3860</v>
       </c>
@@ -33203,7 +33203,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="241">
         <v>3861</v>
       </c>
@@ -33223,7 +33223,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="241" t="s">
         <v>1045</v>
       </c>
@@ -33243,7 +33243,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="241" t="s">
         <v>1046</v>
       </c>
@@ -33263,7 +33263,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="241">
         <v>3865</v>
       </c>
@@ -33283,7 +33283,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="241">
         <v>3869</v>
       </c>
@@ -33303,7 +33303,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="241">
         <v>3870</v>
       </c>
@@ -33321,7 +33321,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="241" t="s">
         <v>1047</v>
       </c>
@@ -33341,7 +33341,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="241" t="s">
         <v>1048</v>
       </c>
@@ -33361,7 +33361,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="241">
         <v>3877</v>
       </c>
@@ -33381,7 +33381,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="241">
         <v>3878</v>
       </c>
@@ -33401,7 +33401,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="241">
         <v>3879</v>
       </c>
@@ -33421,7 +33421,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="35" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="241">
         <v>3880</v>
       </c>
@@ -33441,7 +33441,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="243" t="s">
         <v>1424</v>
       </c>
@@ -33461,7 +33461,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="243" t="s">
         <v>1422</v>
       </c>
@@ -33481,7 +33481,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="242">
         <v>3883</v>
       </c>
@@ -33501,7 +33501,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="244">
         <v>3886</v>
       </c>
@@ -33521,7 +33521,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="242">
         <v>3888</v>
       </c>
@@ -33541,7 +33541,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="242">
         <v>3889</v>
       </c>
@@ -33561,7 +33561,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="42" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="242">
         <v>3891</v>
       </c>
@@ -33581,7 +33581,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="43" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="242" t="s">
         <v>1049</v>
       </c>
@@ -33601,7 +33601,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="44" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="242" t="s">
         <v>1050</v>
       </c>
@@ -33621,7 +33621,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="45" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="242">
         <v>3893</v>
       </c>
@@ -33641,7 +33641,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="242">
         <v>3896</v>
       </c>
@@ -33661,7 +33661,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="242">
         <v>3897</v>
       </c>
@@ -33681,7 +33681,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="242">
         <v>3898</v>
       </c>
@@ -33701,7 +33701,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="49" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="242" t="s">
         <v>1051</v>
       </c>
@@ -33721,7 +33721,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="242" t="s">
         <v>1052</v>
       </c>
@@ -33741,7 +33741,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="51" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="242">
         <v>3150</v>
       </c>
@@ -33761,7 +33761,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="52" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="245" t="s">
         <v>1083</v>
       </c>
@@ -33781,7 +33781,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="53" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="245" t="s">
         <v>1084</v>
       </c>
@@ -33801,7 +33801,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="54" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="246" t="s">
         <v>1085</v>
       </c>
@@ -33821,7 +33821,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="19.2" customHeight="1" ns3:dyDescent="0.3">
+    <row r="55" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="246" t="s">
         <v>1086</v>
       </c>
@@ -33839,7 +33839,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="56" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="242">
         <v>3633</v>
       </c>
@@ -33859,7 +33859,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="57" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="242">
         <v>3802</v>
       </c>
@@ -33879,7 +33879,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="58" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="242">
         <v>3862</v>
       </c>
@@ -33899,7 +33899,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="59" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="242" t="s">
         <v>1427</v>
       </c>
@@ -33919,7 +33919,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="60" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="242" t="s">
         <v>1428</v>
       </c>
@@ -33939,7 +33939,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="61" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="242" t="s">
         <v>1429</v>
       </c>
@@ -33959,7 +33959,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="62" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="242" t="s">
         <v>1430</v>
       </c>
@@ -33979,7 +33979,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="63" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="242">
         <v>3880</v>
       </c>
@@ -33999,7 +33999,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="64" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="242">
         <v>3882</v>
       </c>
@@ -34019,7 +34019,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="65" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="242">
         <v>3894</v>
       </c>
@@ -34039,7 +34039,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="66" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="242">
         <v>3902</v>
       </c>
@@ -34059,7 +34059,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="67" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="242">
         <v>3904</v>
       </c>
@@ -34079,7 +34079,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="68" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="242">
         <v>3905</v>
       </c>
@@ -34099,7 +34099,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="69" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="242">
         <v>3906</v>
       </c>
@@ -34119,7 +34119,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="70" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="242">
         <v>3915</v>
       </c>
@@ -34139,7 +34139,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="71" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="242" t="s">
         <v>1431</v>
       </c>
@@ -34159,7 +34159,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="72" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="242" t="s">
         <v>1432</v>
       </c>
@@ -34179,7 +34179,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="73" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="242">
         <v>3921</v>
       </c>
@@ -34199,7 +34199,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="74" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="242">
         <v>3922</v>
       </c>
@@ -34219,7 +34219,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="75" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="242">
         <v>3932</v>
       </c>
@@ -34239,7 +34239,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="76" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="242">
         <v>3937</v>
       </c>
@@ -34259,7 +34259,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="77" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="242">
         <v>3940</v>
       </c>
@@ -34279,7 +34279,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="78" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="242">
         <v>3941</v>
       </c>
@@ -34299,7 +34299,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="79" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="242">
         <v>3944</v>
       </c>
@@ -34319,7 +34319,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="80" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="242">
         <v>3947</v>
       </c>
@@ -34339,7 +34339,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="81" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="242" t="s">
         <v>1433</v>
       </c>
@@ -34359,7 +34359,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="82" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="242" t="s">
         <v>1434</v>
       </c>
@@ -34379,7 +34379,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="83" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="242" t="s">
         <v>1435</v>
       </c>
@@ -34399,7 +34399,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="84" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="242" t="s">
         <v>1436</v>
       </c>
@@ -34419,7 +34419,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="85" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="242" t="s">
         <v>1437</v>
       </c>
@@ -34439,7 +34439,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="86" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="242" t="s">
         <v>1438</v>
       </c>
@@ -34459,7 +34459,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="87" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="242">
         <v>3955</v>
       </c>
@@ -34479,7 +34479,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="88" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="242">
         <v>3957</v>
       </c>
@@ -34499,7 +34499,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="89" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="242" t="s">
         <v>1439</v>
       </c>
@@ -34519,7 +34519,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="90" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="242" t="s">
         <v>1440</v>
       </c>
@@ -34539,7 +34539,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="91" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="242" t="s">
         <v>1441</v>
       </c>
@@ -34559,7 +34559,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="92" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="242" t="s">
         <v>1442</v>
       </c>
@@ -34579,7 +34579,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="93" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="242">
         <v>3961</v>
       </c>
@@ -34599,7 +34599,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="94" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="242">
         <v>3962</v>
       </c>
@@ -34619,7 +34619,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="95" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="242" t="s">
         <v>1443</v>
       </c>
@@ -34639,7 +34639,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="96" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="242">
         <v>3967</v>
       </c>
@@ -34659,7 +34659,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="97" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="97" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="242">
         <v>3968</v>
       </c>
@@ -34679,7 +34679,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="98" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="98" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="242" t="s">
         <v>1444</v>
       </c>
@@ -34699,7 +34699,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="99" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="99" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="242" t="s">
         <v>1445</v>
       </c>
@@ -34719,7 +34719,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="100" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="242" t="s">
         <v>1446</v>
       </c>
@@ -34739,7 +34739,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="101" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="242" t="s">
         <v>1447</v>
       </c>
@@ -34759,7 +34759,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="102" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="242" t="s">
         <v>1448</v>
       </c>
@@ -34779,7 +34779,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="103" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="103" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="242">
         <v>3972</v>
       </c>
@@ -34799,7 +34799,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="104" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="104" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="242">
         <v>3984</v>
       </c>
@@ -34819,7 +34819,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="105" spans="1:12" ht="17.399999999999999" customHeight="1" ns3:dyDescent="0.3">
+    <row r="105" spans="1:12" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="242">
         <v>3985</v>
       </c>
@@ -34839,7 +34839,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="106" spans="1:12" ht="17.399999999999999" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="106" spans="1:12" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A106" s="242">
         <v>3990</v>
       </c>
@@ -34859,7 +34859,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="107" spans="1:12" ns3:dyDescent="0.3">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107" s="247">
         <v>4001</v>
       </c>
@@ -34891,7 +34891,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="108" spans="1:12" ns3:dyDescent="0.3">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" s="248">
         <v>4003</v>
       </c>
@@ -34924,7 +34924,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="109" spans="1:12" ns3:dyDescent="0.3">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A109" s="248">
         <v>4008</v>
       </c>
@@ -34957,7 +34957,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="110" spans="1:12" ns3:dyDescent="0.3">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A110" s="248">
         <v>4009</v>
       </c>
@@ -34989,7 +34989,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="111" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="111" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="248">
         <v>4010</v>
       </c>
@@ -35021,7 +35021,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="112" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="112" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="248">
         <v>4013</v>
       </c>
@@ -35053,7 +35053,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="113" spans="1:12" ns3:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" s="248">
         <v>4018</v>
       </c>
@@ -35085,7 +35085,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="114" spans="1:12" ns3:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114" s="248">
         <v>4019</v>
       </c>
@@ -35115,7 +35115,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="115" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="115" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A115" s="232">
         <v>4019</v>
       </c>
@@ -35147,7 +35147,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="116" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="116" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="249">
         <v>4024</v>
       </c>
@@ -35171,7 +35171,7 @@
       <c r="K116" s="157"/>
       <c r="L116" s="158"/>
     </row>
-    <row r="117" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="117" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="249">
         <v>4026</v>
       </c>
@@ -35201,7 +35201,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="118" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="118" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="250">
         <v>4028</v>
       </c>
@@ -35233,7 +35233,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="119" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="119" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A119" s="250">
         <v>4033</v>
       </c>
@@ -35263,7 +35263,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="120" spans="1:12" ns3:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120" s="251">
         <v>4034</v>
       </c>
@@ -35287,7 +35287,7 @@
       <c r="K120" s="161"/>
       <c r="L120" s="162"/>
     </row>
-    <row r="121" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="121" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A121" s="248">
         <v>4035</v>
       </c>
@@ -35319,7 +35319,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="122" spans="1:12" ns3:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" s="248">
         <v>4036</v>
       </c>
@@ -35349,7 +35349,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="123" spans="1:12" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="123" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A123" s="252">
         <v>4042</v>
       </c>
@@ -35381,7 +35381,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="124" spans="1:12" ns3:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124" s="253">
         <v>4044</v>
       </c>
@@ -35411,7 +35411,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="125" spans="1:12" ns3:dyDescent="0.3">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A125" s="233">
         <v>4044</v>
       </c>
@@ -35435,7 +35435,7 @@
       <c r="K125" s="161"/>
       <c r="L125" s="162"/>
     </row>
-    <row r="126" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="126" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="233">
         <v>4044</v>
       </c>
@@ -35467,7 +35467,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="127" spans="1:12" ns3:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127" s="254">
         <v>4051</v>
       </c>
@@ -35499,7 +35499,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="128" spans="1:12" ns3:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128" s="254">
         <v>4052</v>
       </c>
@@ -35531,7 +35531,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="129" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="129" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A129" s="255">
         <v>4053</v>
       </c>
@@ -35563,7 +35563,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="130" spans="1:12" ns3:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A130" s="256">
         <v>4053</v>
       </c>
@@ -35585,7 +35585,7 @@
       <c r="K130" s="153"/>
       <c r="L130" s="154"/>
     </row>
-    <row r="131" spans="1:12" ns3:dyDescent="0.3">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A131" s="257">
         <v>4056</v>
       </c>
@@ -35617,7 +35617,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="132" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="132" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="234">
         <v>4060</v>
       </c>
@@ -35643,7 +35643,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ns3:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A133" s="258">
         <v>4061</v>
       </c>
@@ -35675,7 +35675,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="134" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="134" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="233">
         <v>4061</v>
       </c>
@@ -35699,7 +35699,7 @@
       <c r="K134" s="153"/>
       <c r="L134" s="154"/>
     </row>
-    <row r="135" spans="1:12" ns3:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A135" s="259">
         <v>4064</v>
       </c>
@@ -35731,7 +35731,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="136" spans="1:12" ns3:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A136" s="259">
         <v>4065</v>
       </c>
@@ -35761,7 +35761,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="137" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="137" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="233">
         <v>4065</v>
       </c>
@@ -35793,7 +35793,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="138" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="138" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="233">
         <v>4076</v>
       </c>
@@ -35825,7 +35825,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="139" spans="1:12" ns3:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A139" s="259" t="s">
         <v>1492</v>
       </c>
@@ -35857,7 +35857,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="140" spans="1:12" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="140" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A140" s="259" t="s">
         <v>1492</v>
       </c>
@@ -35887,7 +35887,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="141" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="141" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="233" t="s">
         <v>1492</v>
       </c>
@@ -35919,7 +35919,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="142" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="142" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="259" t="s">
         <v>1517</v>
       </c>
@@ -35951,7 +35951,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="143" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="143" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="233" t="s">
         <v>1517</v>
       </c>
@@ -35975,7 +35975,7 @@
       <c r="K143" s="194"/>
       <c r="L143" s="195"/>
     </row>
-    <row r="144" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="144" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A144" s="259" t="s">
         <v>1493</v>
       </c>
@@ -36005,7 +36005,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="145" spans="1:12" ns3:dyDescent="0.3">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A145" s="259" t="s">
         <v>1520</v>
       </c>
@@ -36037,7 +36037,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="146" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="146" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="233" t="s">
         <v>1520</v>
       </c>
@@ -36061,7 +36061,7 @@
       <c r="K146" s="172"/>
       <c r="L146" s="173"/>
     </row>
-    <row r="147" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="147" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="259" t="s">
         <v>1521</v>
       </c>
@@ -36093,7 +36093,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="148" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="148" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="233" t="s">
         <v>1521</v>
       </c>
@@ -36125,7 +36125,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="149" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="149" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="259" t="s">
         <v>1636</v>
       </c>
@@ -36157,7 +36157,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ns3:dyDescent="0.3">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A150" s="233" t="s">
         <v>1495</v>
       </c>
@@ -36189,7 +36189,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="151" spans="1:12" ht="16.2" thickBot="1" ns3:dyDescent="0.35">
+    <row r="151" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A151" s="259" t="s">
         <v>1495</v>
       </c>
@@ -36219,7 +36219,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="152" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="152" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="233" t="s">
         <v>1495</v>
       </c>
@@ -36251,7 +36251,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="153" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="153" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="259" t="s">
         <v>1601</v>
       </c>
@@ -36283,7 +36283,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="154" spans="1:12" ns3:dyDescent="0.3">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A154" s="259" t="s">
         <v>1507</v>
       </c>
@@ -36315,7 +36315,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="155" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="155" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A155" s="259" t="s">
         <v>1603</v>
       </c>
@@ -36347,7 +36347,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="156" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="156" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="260" t="s">
         <v>1633</v>
       </c>
@@ -36379,7 +36379,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="157" spans="1:12" ns3:dyDescent="0.3">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157" s="260" t="s">
         <v>1528</v>
       </c>
@@ -36411,7 +36411,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="158" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="158" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="261" t="s">
         <v>1528</v>
       </c>
@@ -36443,7 +36443,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="159" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="159" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="259" t="s">
         <v>1526</v>
       </c>
@@ -36475,7 +36475,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="160" spans="1:12" ns3:dyDescent="0.3">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A160" s="259" t="s">
         <v>1525</v>
       </c>
@@ -36507,7 +36507,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="161" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="161" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="259" t="s">
         <v>1496</v>
       </c>
@@ -36539,7 +36539,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="162" spans="1:12" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="162" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="259" t="s">
         <v>1630</v>
       </c>
@@ -36571,7 +36571,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="163" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="163" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="259" t="s">
         <v>1631</v>
       </c>
@@ -36603,7 +36603,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="164" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="164" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="260" t="s">
         <v>1499</v>
       </c>
@@ -36635,7 +36635,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="165" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="165" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="235" t="s">
         <v>1576</v>
       </c>
@@ -36667,7 +36667,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="166" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="166" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="260" t="s">
         <v>1500</v>
       </c>
@@ -36699,7 +36699,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="167" spans="1:12" ns3:dyDescent="0.3">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A167" s="259" t="s">
         <v>1625</v>
       </c>
@@ -36731,7 +36731,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="168" spans="1:12" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="168" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="233" t="s">
         <v>1501</v>
       </c>
@@ -36763,7 +36763,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="169" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="169" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="259" t="s">
         <v>1627</v>
       </c>
@@ -36783,7 +36783,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="170" spans="1:12" ns3:dyDescent="0.3">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A170" s="259" t="s">
         <v>1628</v>
       </c>
@@ -36803,7 +36803,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="171" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="171" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="233" t="s">
         <v>1557</v>
       </c>
@@ -36823,7 +36823,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="172" spans="1:12" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="172" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="233" t="s">
         <v>1556</v>
       </c>
@@ -36843,7 +36843,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="173" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="173" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="259" t="s">
         <v>1551</v>
       </c>
@@ -36863,7 +36863,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="174" spans="1:12" ns3:dyDescent="0.3">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A174" s="259" t="s">
         <v>1538</v>
       </c>
@@ -36883,7 +36883,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="175" spans="1:12" ht="16.5" customHeight="1" ns3:dyDescent="0.3">
+    <row r="175" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="259" t="s">
         <v>1609</v>
       </c>
@@ -36903,7 +36903,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="176" spans="1:12" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="176" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="259" t="s">
         <v>1610</v>
       </c>
@@ -36923,7 +36923,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="177" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="233" t="s">
         <v>1613</v>
       </c>
@@ -36943,7 +36943,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ns3:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="262" t="s">
         <v>1489</v>
       </c>
@@ -36961,7 +36961,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="179" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="233" t="s">
         <v>1572</v>
       </c>
@@ -36981,7 +36981,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.25">
+    <row r="180" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="236" t="s">
         <v>1566</v>
       </c>
@@ -37001,7 +37001,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="181" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="259" t="s">
         <v>1604</v>
       </c>
@@ -37021,7 +37021,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="16.5" customHeight="1" ns3:dyDescent="0.3">
+    <row r="182" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="259" t="s">
         <v>1605</v>
       </c>
@@ -37041,7 +37041,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ns3:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="259" t="s">
         <v>1505</v>
       </c>
@@ -37061,7 +37061,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ns3:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="259" t="s">
         <v>1505</v>
       </c>
@@ -37081,7 +37081,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="185" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="259" t="s">
         <v>1574</v>
       </c>
@@ -37101,7 +37101,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="186" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="259" t="s">
         <v>1574</v>
       </c>
@@ -37121,7 +37121,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ns3:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" s="233" t="s">
         <v>1593</v>
       </c>
@@ -37141,7 +37141,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ns3:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="236" t="s">
         <v>1568</v>
       </c>
@@ -37161,7 +37161,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ns3:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="236" t="s">
         <v>1570</v>
       </c>
@@ -37181,7 +37181,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="190" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="233" t="s">
         <v>1592</v>
       </c>
@@ -37201,7 +37201,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="191" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="233" t="s">
         <v>1581</v>
       </c>
@@ -37221,7 +37221,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="192" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="233" t="s">
         <v>1581</v>
       </c>
@@ -37241,7 +37241,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="193" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="233" t="s">
         <v>1582</v>
       </c>
@@ -37261,7 +37261,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="194" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="194" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="233" t="s">
         <v>1582</v>
       </c>
@@ -37281,7 +37281,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ns3:dyDescent="0.3">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="259" t="s">
         <v>1497</v>
       </c>
@@ -37301,7 +37301,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="196" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="196" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="233" t="s">
         <v>1619</v>
       </c>
@@ -37321,7 +37321,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ns3:dyDescent="0.3">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="259" t="s">
         <v>1498</v>
       </c>
@@ -37339,7 +37339,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="198" spans="1:6" ns3:dyDescent="0.3">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" s="233" t="s">
         <v>1622</v>
       </c>
@@ -37359,7 +37359,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="199" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="199" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="259" t="s">
         <v>1490</v>
       </c>
@@ -37379,7 +37379,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="200" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="200" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="263" t="s">
         <v>1598</v>
       </c>
@@ -37399,7 +37399,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="201" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
+    <row r="201" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="263" t="s">
         <v>1550</v>
       </c>
@@ -37419,7 +37419,7 @@
         <v>25991</v>
       </c>
     </row>
-    <row r="202" spans="1:6" ns3:dyDescent="0.3">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" s="237" t="s">
         <v>1585</v>
       </c>
@@ -37439,7 +37439,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="203" spans="1:6" ns3:dyDescent="0.3">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="237" t="s">
         <v>1584</v>
       </c>
@@ -37459,7 +37459,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="204" spans="1:6" ns3:dyDescent="0.3">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" s="237" t="s">
         <v>1588</v>
       </c>
@@ -37479,7 +37479,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="205" spans="1:6" ns3:dyDescent="0.3">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="237" t="s">
         <v>1616</v>
       </c>
@@ -37499,7 +37499,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="206" spans="1:6" ns3:dyDescent="0.3">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" s="237" t="s">
         <v>1583</v>
       </c>
@@ -37511,7 +37511,7 @@
       <c r="E206" s="179"/>
       <c r="F206" s="29"/>
     </row>
-    <row r="207" spans="1:6" ns3:dyDescent="0.3">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" s="237" t="s">
         <v>1617</v>
       </c>
@@ -37531,7 +37531,7 @@
         <v>28990</v>
       </c>
     </row>
-    <row r="208" spans="1:6" ns3:dyDescent="0.3">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" s="237" t="s">
         <v>1615</v>
       </c>
@@ -37551,7 +37551,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="209" spans="1:6" ns3:dyDescent="0.25">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="238" t="s">
         <v>1579</v>
       </c>
@@ -37571,7 +37571,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="210" spans="1:6" ns3:dyDescent="0.25">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" s="238"/>
       <c r="B210" s="238"/>
       <c r="C210" s="189" t="s">
@@ -37587,7 +37587,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="211" spans="1:6" ns3:dyDescent="0.3">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" s="237" t="s">
         <v>1637</v>
       </c>
@@ -37605,7 +37605,7 @@
       </c>
       <c r="F211" s="29"/>
     </row>
-    <row r="212" spans="1:6" ns3:dyDescent="0.3">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" s="237" t="s">
         <v>1641</v>
       </c>
@@ -37623,7 +37623,7 @@
       </c>
       <c r="F212" s="29"/>
     </row>
-    <row r="213" spans="1:6" ns3:dyDescent="0.3">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213" s="237" t="s">
         <v>1645</v>
       </c>
@@ -37637,7 +37637,7 @@
       <c r="E213" s="179"/>
       <c r="F213" s="29"/>
     </row>
-    <row r="214" spans="1:6" ns3:dyDescent="0.3">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" s="237" t="s">
         <v>1646</v>
       </c>
@@ -37651,7 +37651,7 @@
       <c r="E214" s="179"/>
       <c r="F214" s="29"/>
     </row>
-    <row r="215" spans="1:6" ns3:dyDescent="0.3">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215" s="237" t="s">
         <v>1649</v>
       </c>
@@ -37665,7 +37665,7 @@
       <c r="E215" s="179"/>
       <c r="F215" s="29"/>
     </row>
-    <row r="216" spans="1:6" ns3:dyDescent="0.3">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216" s="237" t="s">
         <v>1650</v>
       </c>
@@ -37679,7 +37679,7 @@
       <c r="E216" s="179"/>
       <c r="F216" s="29"/>
     </row>
-    <row r="217" spans="1:6" ns3:dyDescent="0.3">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" s="237">
         <v>4074</v>
       </c>
@@ -37695,7 +37695,7 @@
       <c r="E217" s="179"/>
       <c r="F217" s="29"/>
     </row>
-    <row r="218" spans="1:6" ns3:dyDescent="0.25">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" s="223">
         <v>4101</v>
       </c>
@@ -37715,7 +37715,7 @@
         <v>20990</v>
       </c>
     </row>
-    <row r="219" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.3">
+    <row r="219" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="237" t="s">
         <v>1759</v>
       </c>
@@ -37735,7 +37735,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="220" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="220" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="238" t="s">
         <v>1676</v>
       </c>
@@ -37755,7 +37755,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="221" spans="1:6" ns3:dyDescent="0.3">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221" s="237" t="s">
         <v>1757</v>
       </c>
@@ -37775,7 +37775,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="222" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="222" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="238" t="s">
         <v>1737</v>
       </c>
@@ -37795,7 +37795,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="223" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="223" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="238" t="s">
         <v>1679</v>
       </c>
@@ -37815,7 +37815,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="224" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="224" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="238" t="s">
         <v>1701</v>
       </c>
@@ -37835,7 +37835,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="225" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="225" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="238" t="s">
         <v>1704</v>
       </c>
@@ -37855,7 +37855,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="226" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="226" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="238" t="s">
         <v>1720</v>
       </c>
@@ -37875,7 +37875,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="227" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="227" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="238" t="s">
         <v>1719</v>
       </c>
@@ -37895,7 +37895,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="228" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="228" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="238" t="s">
         <v>1664</v>
       </c>
@@ -37915,7 +37915,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="229" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="229" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="238" t="s">
         <v>1724</v>
       </c>
@@ -37935,7 +37935,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="230" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="230" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="238" t="s">
         <v>1694</v>
       </c>
@@ -37955,7 +37955,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="231" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="231" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="238" t="s">
         <v>1694</v>
       </c>
@@ -37975,7 +37975,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="232" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="232" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="238" t="s">
         <v>1696</v>
       </c>
@@ -37995,7 +37995,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="233" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="233" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="238" t="s">
         <v>1673</v>
       </c>
@@ -38015,7 +38015,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="234" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="234" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="238" t="s">
         <v>1733</v>
       </c>
@@ -38035,7 +38035,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="235" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="235" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="238" t="s">
         <v>1717</v>
       </c>
@@ -38055,7 +38055,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="236" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="236" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="238" t="s">
         <v>1668</v>
       </c>
@@ -38075,7 +38075,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="237" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="237" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="238" t="s">
         <v>1668</v>
       </c>
@@ -38095,7 +38095,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="238" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="238" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="238" t="s">
         <v>1715</v>
       </c>
@@ -38115,7 +38115,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="239" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="239" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="238" t="s">
         <v>1670</v>
       </c>
@@ -38135,7 +38135,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="240" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="240" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="238" t="s">
         <v>1693</v>
       </c>
@@ -38155,7 +38155,7 @@
         <v>21990</v>
       </c>
     </row>
-    <row r="241" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="241" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="238" t="s">
         <v>1688</v>
       </c>
@@ -38175,7 +38175,7 @@
         <v>23990</v>
       </c>
     </row>
-    <row r="242" spans="1:6" ns3:dyDescent="0.25">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242" s="223">
         <v>4106</v>
       </c>
@@ -38195,7 +38195,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="243" spans="1:6" ns3:dyDescent="0.25">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" s="223">
         <v>4108</v>
       </c>
@@ -38215,7 +38215,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="244" spans="1:6" ns3:dyDescent="0.25">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" s="223">
         <v>4108</v>
       </c>
@@ -38235,7 +38235,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="245" spans="1:6" ns3:dyDescent="0.25">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="223">
         <v>4109</v>
       </c>
@@ -38255,7 +38255,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="246" spans="1:6" ns3:dyDescent="0.25">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" s="223">
         <v>4109</v>
       </c>
@@ -38275,7 +38275,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="247" spans="1:6" ns3:dyDescent="0.25">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" s="223">
         <v>4110</v>
       </c>
@@ -38295,7 +38295,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="248" spans="1:6" ns3:dyDescent="0.25">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248" s="223">
         <v>4113</v>
       </c>
@@ -38315,7 +38315,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="249" spans="1:6" ns3:dyDescent="0.25">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" s="223">
         <v>4113</v>
       </c>
@@ -38335,7 +38335,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="250" spans="1:6" ns3:dyDescent="0.25">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" s="223">
         <v>4116</v>
       </c>
@@ -38355,7 +38355,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="251" spans="1:6" ns3:dyDescent="0.25">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="223">
         <v>4119</v>
       </c>
@@ -38375,7 +38375,7 @@
         <v>21990</v>
       </c>
     </row>
-    <row r="252" spans="1:6" ns3:dyDescent="0.25">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" s="223">
         <v>4120</v>
       </c>
@@ -38395,7 +38395,7 @@
         <v>20990</v>
       </c>
     </row>
-    <row r="253" spans="1:6" ns3:dyDescent="0.25">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" s="223">
         <v>4121</v>
       </c>
@@ -38415,7 +38415,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="254" spans="1:6" ns3:dyDescent="0.25">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" s="223">
         <v>4122</v>
       </c>
@@ -38435,7 +38435,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="255" spans="1:6" ns3:dyDescent="0.25">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" s="223">
         <v>4123</v>
       </c>
@@ -38455,7 +38455,7 @@
         <v>20990</v>
       </c>
     </row>
-    <row r="256" spans="1:6" ns3:dyDescent="0.25">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" s="223" t="s">
         <v>1743</v>
       </c>
@@ -38475,7 +38475,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="257" spans="1:18" ns3:dyDescent="0.25">
+    <row r="257" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A257" s="223">
         <v>4128</v>
       </c>
@@ -38495,7 +38495,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="258" spans="1:18" ns3:dyDescent="0.25">
+    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A258" s="223">
         <v>4130</v>
       </c>
@@ -38515,7 +38515,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ns3:dyDescent="0.25">
+    <row r="259" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A259" s="223">
         <v>4135</v>
       </c>
@@ -38535,7 +38535,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="260" spans="1:18" ns3:dyDescent="0.25">
+    <row r="260" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A260" s="223">
         <v>4136</v>
       </c>
@@ -38555,7 +38555,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="261" spans="1:18" ns3:dyDescent="0.25">
+    <row r="261" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A261" s="223">
         <v>4137</v>
       </c>
@@ -38575,7 +38575,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="262" spans="1:18" ns3:dyDescent="0.25">
+    <row r="262" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A262" s="223">
         <v>4149</v>
       </c>
@@ -38595,7 +38595,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="263" spans="1:18" ns3:dyDescent="0.25">
+    <row r="263" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A263" s="223">
         <v>4153</v>
       </c>
@@ -38615,7 +38615,7 @@
         <v>21990</v>
       </c>
     </row>
-    <row r="264" spans="1:18" ns3:dyDescent="0.25">
+    <row r="264" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A264" s="223" t="s">
         <v>1747</v>
       </c>
@@ -38635,7 +38635,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="265" spans="1:18" ns3:dyDescent="0.25">
+    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A265" s="223" t="s">
         <v>1748</v>
       </c>
@@ -38655,7 +38655,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="266" spans="1:18" ns3:dyDescent="0.25">
+    <row r="266" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A266" s="223">
         <v>4158</v>
       </c>
@@ -38675,7 +38675,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="267" spans="1:18" ns3:dyDescent="0.25">
+    <row r="267" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A267" s="223">
         <v>4160</v>
       </c>
@@ -38695,7 +38695,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="268" spans="1:18" ns3:dyDescent="0.25">
+    <row r="268" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A268" s="223">
         <v>4165</v>
       </c>
@@ -38715,7 +38715,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ns3:dyDescent="0.25">
+    <row r="269" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A269" s="223">
         <v>4166</v>
       </c>
@@ -38735,7 +38735,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="270" spans="1:18" ns3:dyDescent="0.25">
+    <row r="270" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A270" s="223">
         <v>4166</v>
       </c>
@@ -38763,7 +38763,7 @@
       <c r="Q270" s="216"/>
       <c r="R270" s="216"/>
     </row>
-    <row r="271" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="271" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A271" s="221">
         <v>4168</v>
       </c>
@@ -38791,7 +38791,7 @@
       <c r="Q271" s="216"/>
       <c r="R271" s="216"/>
     </row>
-    <row r="272" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="272" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A272" s="221">
         <v>4168</v>
       </c>
@@ -38815,7 +38815,7 @@
       <c r="Q272" s="216"/>
       <c r="R272" s="216"/>
     </row>
-    <row r="273" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="273" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A273" s="221">
         <v>4176</v>
       </c>
@@ -38843,7 +38843,7 @@
       <c r="Q273" s="216"/>
       <c r="R273" s="216"/>
     </row>
-    <row r="274" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="274" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A274" s="221">
         <v>4176</v>
       </c>
@@ -38871,7 +38871,7 @@
       <c r="Q274" s="216"/>
       <c r="R274" s="216"/>
     </row>
-    <row r="275" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="275" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A275" s="221">
         <v>4177</v>
       </c>
@@ -38899,7 +38899,7 @@
       <c r="Q275" s="216"/>
       <c r="R275" s="216"/>
     </row>
-    <row r="276" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="276" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A276" s="221">
         <v>4178</v>
       </c>
@@ -38927,7 +38927,7 @@
       <c r="Q276" s="216"/>
       <c r="R276" s="216"/>
     </row>
-    <row r="277" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="277" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A277" s="221">
         <v>4179</v>
       </c>
@@ -38953,7 +38953,7 @@
       <c r="Q277" s="216"/>
       <c r="R277" s="216"/>
     </row>
-    <row r="278" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="278" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A278" s="221">
         <v>4183</v>
       </c>
@@ -38981,7 +38981,7 @@
       <c r="Q278" s="216"/>
       <c r="R278" s="216"/>
     </row>
-    <row r="279" spans="1:18" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="279" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A279" s="269">
         <v>4185</v>
       </c>
@@ -39009,7 +39009,7 @@
       <c r="Q279" s="216"/>
       <c r="R279" s="216"/>
     </row>
-    <row r="280" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.35">
+    <row r="280" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A280" s="264"/>
       <c r="B280" s="264"/>
       <c r="C280" s="277" t="s">
@@ -39027,7 +39027,7 @@
       <c r="Q280" s="216"/>
       <c r="R280" s="216"/>
     </row>
-    <row r="281" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="281" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A281" s="278" t="s">
         <v>1790</v>
       </c>
@@ -39055,7 +39055,7 @@
       <c r="Q281" s="216"/>
       <c r="R281" s="216"/>
     </row>
-    <row r="282" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="282" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="279" t="s">
         <v>1750</v>
       </c>
@@ -39083,7 +39083,7 @@
       <c r="Q282" s="216"/>
       <c r="R282" s="216"/>
     </row>
-    <row r="283" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="283" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A283" s="279" t="s">
         <v>1791</v>
       </c>
@@ -39111,7 +39111,7 @@
       <c r="Q283" s="216"/>
       <c r="R283" s="216"/>
     </row>
-    <row r="284" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="284" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A284" s="279" t="s">
         <v>1769</v>
       </c>
@@ -39139,7 +39139,7 @@
       <c r="Q284" s="216"/>
       <c r="R284" s="216"/>
     </row>
-    <row r="285" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="285" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="279" t="s">
         <v>1792</v>
       </c>
@@ -39167,7 +39167,7 @@
       <c r="Q285" s="216"/>
       <c r="R285" s="216"/>
     </row>
-    <row r="286" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="286" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A286" s="279" t="s">
         <v>1774</v>
       </c>
@@ -39195,7 +39195,7 @@
       <c r="Q286" s="216"/>
       <c r="R286" s="216"/>
     </row>
-    <row r="287" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="287" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A287" s="279" t="s">
         <v>1756</v>
       </c>
@@ -39223,7 +39223,7 @@
       <c r="Q287" s="216"/>
       <c r="R287" s="216"/>
     </row>
-    <row r="288" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="288" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A288" s="279" t="s">
         <v>1794</v>
       </c>
@@ -39251,7 +39251,7 @@
       <c r="Q288" s="216"/>
       <c r="R288" s="216"/>
     </row>
-    <row r="289" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="289" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="279" t="s">
         <v>1785</v>
       </c>
@@ -39279,7 +39279,7 @@
       <c r="Q289" s="216"/>
       <c r="R289" s="216"/>
     </row>
-    <row r="290" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="290" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A290" s="279" t="s">
         <v>1787</v>
       </c>
@@ -39307,7 +39307,7 @@
       <c r="Q290" s="216"/>
       <c r="R290" s="216"/>
     </row>
-    <row r="291" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="291" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A291" s="279" t="s">
         <v>1755</v>
       </c>
@@ -39335,7 +39335,7 @@
       <c r="Q291" s="216"/>
       <c r="R291" s="216"/>
     </row>
-    <row r="292" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="292" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A292" s="279" t="s">
         <v>1795</v>
       </c>
@@ -39363,7 +39363,7 @@
       <c r="Q292" s="216"/>
       <c r="R292" s="216"/>
     </row>
-    <row r="293" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="293" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="279" t="s">
         <v>1796</v>
       </c>
@@ -39391,7 +39391,7 @@
       <c r="Q293" s="216"/>
       <c r="R293" s="216"/>
     </row>
-    <row r="294" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="294" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A294" s="279" t="s">
         <v>2094</v>
       </c>
@@ -39419,7 +39419,7 @@
       <c r="Q294" s="216"/>
       <c r="R294" s="216"/>
     </row>
-    <row r="295" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="295" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A295" s="279" t="s">
         <v>2112</v>
       </c>
@@ -39447,7 +39447,7 @@
       <c r="Q295" s="216"/>
       <c r="R295" s="216"/>
     </row>
-    <row r="296" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="296" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="279" t="s">
         <v>1762</v>
       </c>
@@ -39475,7 +39475,7 @@
       <c r="Q296" s="216"/>
       <c r="R296" s="216"/>
     </row>
-    <row r="297" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="297" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A297" s="279" t="s">
         <v>1797</v>
       </c>
@@ -39503,7 +39503,7 @@
       <c r="Q297" s="216"/>
       <c r="R297" s="216"/>
     </row>
-    <row r="298" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="298" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A298" s="279" t="s">
         <v>1751</v>
       </c>
@@ -39531,7 +39531,7 @@
       <c r="Q298" s="216"/>
       <c r="R298" s="216"/>
     </row>
-    <row r="299" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="299" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="279" t="s">
         <v>1786</v>
       </c>
@@ -39559,7 +39559,7 @@
       <c r="Q299" s="216"/>
       <c r="R299" s="216"/>
     </row>
-    <row r="300" spans="1:18" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="300" spans="1:18" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A300" s="279" t="s">
         <v>1754</v>
       </c>
@@ -39587,7 +39587,7 @@
       <c r="Q300" s="216"/>
       <c r="R300" s="216"/>
     </row>
-    <row r="301" spans="1:18" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="301" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A301" s="279" t="s">
         <v>1798</v>
       </c>
@@ -39615,7 +39615,7 @@
       <c r="Q301" s="215"/>
       <c r="R301" s="215"/>
     </row>
-    <row r="302" spans="1:18" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="302" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A302" s="279" t="s">
         <v>1788</v>
       </c>
@@ -39635,7 +39635,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="303" spans="1:18" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="303" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A303" s="279" t="s">
         <v>1768</v>
       </c>
@@ -39655,7 +39655,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="304" spans="1:18" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="304" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A304" s="279" t="s">
         <v>1799</v>
       </c>
@@ -39675,7 +39675,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="305" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="305" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A305" s="279" t="s">
         <v>1767</v>
       </c>
@@ -39695,7 +39695,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="306" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="306" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="279" t="s">
         <v>1800</v>
       </c>
@@ -39715,7 +39715,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="307" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="307" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A307" s="279" t="s">
         <v>1801</v>
       </c>
@@ -39735,7 +39735,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="308" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="308" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="279" t="s">
         <v>1802</v>
       </c>
@@ -39755,7 +39755,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="309" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="309" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="279" t="s">
         <v>1752</v>
       </c>
@@ -39775,7 +39775,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="310" spans="1:6" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="310" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="279" t="s">
         <v>1753</v>
       </c>
@@ -39795,7 +39795,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="311" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="311" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A311" s="279" t="s">
         <v>2113</v>
       </c>
@@ -39815,7 +39815,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="312" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="312" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A312" s="279" t="s">
         <v>1803</v>
       </c>
@@ -39835,7 +39835,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="313" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="313" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A313" s="279" t="s">
         <v>1775</v>
       </c>
@@ -39855,7 +39855,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="314" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="314" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A314" s="279" t="s">
         <v>1804</v>
       </c>
@@ -39875,7 +39875,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="315" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="315" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A315" s="279" t="s">
         <v>1805</v>
       </c>
@@ -39895,7 +39895,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="316" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="316" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A316" s="279" t="s">
         <v>1806</v>
       </c>
@@ -39915,7 +39915,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="317" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="317" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A317" s="279" t="s">
         <v>1761</v>
       </c>
@@ -39935,7 +39935,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="318" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="318" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A318" s="279" t="s">
         <v>1807</v>
       </c>
@@ -39955,7 +39955,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="319" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="319" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A319" s="279">
         <v>4223</v>
       </c>
@@ -39975,7 +39975,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="320" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="320" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A320" s="279" t="s">
         <v>1808</v>
       </c>
@@ -39995,7 +39995,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="321" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="321" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A321" s="279" t="s">
         <v>1809</v>
       </c>
@@ -40015,7 +40015,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="322" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="322" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A322" s="279" t="s">
         <v>2107</v>
       </c>
@@ -40035,7 +40035,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="323" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="323" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A323" s="279" t="s">
         <v>2106</v>
       </c>
@@ -40055,7 +40055,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="324" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="324" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A324" s="279">
         <v>4226</v>
       </c>
@@ -40075,7 +40075,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="325" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="325" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A325" s="279" t="s">
         <v>2115</v>
       </c>
@@ -40095,7 +40095,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="326" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="326" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A326" s="279" t="s">
         <v>1810</v>
       </c>
@@ -40115,7 +40115,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="327" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="327" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A327" s="279" t="s">
         <v>1812</v>
       </c>
@@ -40135,7 +40135,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="328" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="328" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A328" s="279">
         <v>4228</v>
       </c>
@@ -40155,7 +40155,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="329" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="329" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A329" s="279">
         <v>4229</v>
       </c>
@@ -40175,7 +40175,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="330" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="330" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A330" s="279">
         <v>4230</v>
       </c>
@@ -40195,7 +40195,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="331" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="331" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A331" s="279">
         <v>4232</v>
       </c>
@@ -40215,7 +40215,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="332" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="332" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A332" s="279" t="s">
         <v>1781</v>
       </c>
@@ -40235,7 +40235,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="333" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="333" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A333" s="279" t="s">
         <v>1813</v>
       </c>
@@ -40255,7 +40255,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="334" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="334" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A334" s="279" t="s">
         <v>1782</v>
       </c>
@@ -40275,7 +40275,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="335" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="335" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A335" s="279" t="s">
         <v>1783</v>
       </c>
@@ -40295,7 +40295,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="336" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="336" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A336" s="279" t="s">
         <v>1784</v>
       </c>
@@ -40315,7 +40315,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="337" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="337" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A337" s="279" t="s">
         <v>1814</v>
       </c>
@@ -40335,7 +40335,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="338" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="338" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A338" s="279" t="s">
         <v>1779</v>
       </c>
@@ -40355,7 +40355,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="339" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="339" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A339" s="279" t="s">
         <v>1777</v>
       </c>
@@ -40375,7 +40375,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="340" spans="1:6" ht="16.2" thickBot="1" ns3:dyDescent="0.3">
+    <row r="340" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A340" s="279" t="s">
         <v>1778</v>
       </c>
@@ -40395,7 +40395,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="341" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="341" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A341" s="279" t="s">
         <v>1770</v>
       </c>
@@ -40415,7 +40415,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="342" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="342" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A342" s="279" t="s">
         <v>1815</v>
       </c>
@@ -40435,7 +40435,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="343" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="343" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A343" s="279" t="s">
         <v>2110</v>
       </c>
@@ -40455,7 +40455,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="344" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="344" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A344" s="279" t="s">
         <v>1816</v>
       </c>
@@ -40475,7 +40475,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="345" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="345" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A345" s="279" t="s">
         <v>1817</v>
       </c>
@@ -40495,7 +40495,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="346" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="346" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A346" s="279" t="s">
         <v>1818</v>
       </c>
@@ -40515,7 +40515,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="347" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="347" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A347" s="279" t="s">
         <v>1819</v>
       </c>
@@ -40535,7 +40535,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="348" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="348" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A348" s="279" t="s">
         <v>1820</v>
       </c>
@@ -40555,7 +40555,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="349" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="349" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A349" s="279" t="s">
         <v>1821</v>
       </c>
@@ -40575,7 +40575,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="350" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="350" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A350" s="279" t="s">
         <v>2102</v>
       </c>
@@ -40595,7 +40595,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="351" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="351" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A351" s="279" t="s">
         <v>1822</v>
       </c>
@@ -40615,7 +40615,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="352" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="352" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A352" s="279" t="s">
         <v>1823</v>
       </c>
@@ -40635,7 +40635,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="353" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="353" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A353" s="279" t="s">
         <v>1824</v>
       </c>
@@ -40655,7 +40655,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="354" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="354" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A354" s="279" t="s">
         <v>1825</v>
       </c>
@@ -40675,7 +40675,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="355" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="355" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A355" s="279" t="s">
         <v>1826</v>
       </c>
@@ -40695,7 +40695,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="356" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="356" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A356" s="279" t="s">
         <v>1776</v>
       </c>
@@ -40715,7 +40715,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="357" spans="1:6" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="357" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A357" s="279" t="s">
         <v>1827</v>
       </c>
@@ -40735,7 +40735,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="358" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="358" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A358" s="279" t="s">
         <v>1828</v>
       </c>
@@ -40755,7 +40755,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="359" spans="1:6" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="359" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A359" s="279" t="s">
         <v>1829</v>
       </c>
@@ -40775,7 +40775,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="360" spans="1:6" ht="18" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="360" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A360" s="279" t="s">
         <v>1830</v>
       </c>
@@ -40795,7 +40795,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="361" spans="1:6" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="361" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A361" s="279">
         <v>4256</v>
       </c>
@@ -40815,7 +40815,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="362" spans="1:6" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="362" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A362" s="279" t="s">
         <v>2117</v>
       </c>
@@ -40835,7 +40835,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="363" spans="1:6" ht="16.5" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="363" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A363" s="279" t="s">
         <v>1771</v>
       </c>
@@ -40855,7 +40855,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="364" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="364" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A364" s="279" t="s">
         <v>1772</v>
       </c>
@@ -40875,7 +40875,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="365" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="365" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A365" s="279" t="s">
         <v>1780</v>
       </c>
@@ -40895,7 +40895,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="366" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="366" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A366" s="279" t="s">
         <v>1773</v>
       </c>
@@ -40915,7 +40915,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="367" spans="1:6" ht="15.75" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
+    <row r="367" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A367" s="279" t="s">
         <v>2080</v>
       </c>
@@ -40935,7 +40935,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="368" spans="1:6" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="368" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A368" s="279" t="s">
         <v>2105</v>
       </c>
@@ -40955,7 +40955,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="369" spans="1:9" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="369" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A369" s="179">
         <v>143350038</v>
       </c>
@@ -40981,7 +40981,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="370" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="370" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A370" s="292">
         <v>143110038</v>
       </c>
@@ -41004,7 +41004,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="371" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="371" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A371" s="292">
         <v>143360038</v>
       </c>
@@ -41027,7 +41027,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="372" spans="1:9" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="372" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A372" s="179">
         <v>143560038</v>
       </c>
@@ -41053,7 +41053,7 @@
         <v>2123</v>
       </c>
     </row>
-    <row r="373" spans="1:9" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="373" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A373" s="179">
         <v>143560038</v>
       </c>
@@ -41073,7 +41073,7 @@
         <v>26991</v>
       </c>
     </row>
-    <row r="374" spans="1:9" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="374" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A374" s="290">
         <v>143550038</v>
       </c>
@@ -41087,7 +41087,7 @@
       <c r="E374" s="179"/>
       <c r="F374" s="282"/>
     </row>
-    <row r="375" spans="1:9" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="375" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A375" s="290">
         <v>143530038</v>
       </c>
@@ -41110,7 +41110,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="376" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="376" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A376" s="355">
         <v>143480038</v>
       </c>
@@ -41130,7 +41130,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="377" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="377" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A377" s="360">
         <v>143480038</v>
       </c>
@@ -41150,7 +41150,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="378" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="378" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A378" s="360">
         <v>143486038</v>
       </c>
@@ -41170,7 +41170,7 @@
         <v>24991</v>
       </c>
     </row>
-    <row r="379" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="379" spans="1:9" s="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A379" s="360">
         <v>143480038</v>
       </c>
@@ -41190,7 +41190,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="380" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="380" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A380" s="290">
         <v>143170038</v>
       </c>
@@ -41204,7 +41204,7 @@
       <c r="E380" s="179"/>
       <c r="F380" s="282"/>
     </row>
-    <row r="381" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="381" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A381" s="291">
         <v>143210038</v>
       </c>
@@ -41224,7 +41224,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="382" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="382" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A382" s="291">
         <v>143220038</v>
       </c>
@@ -41244,7 +41244,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="383" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="383" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A383" s="291">
         <v>143220038</v>
       </c>
@@ -41264,7 +41264,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="384" spans="1:9" ht="13.8" ns3:dyDescent="0.25">
+    <row r="384" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A384" s="291">
         <v>143226038</v>
       </c>
@@ -41284,7 +41284,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="385" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="385" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A385" s="291">
         <v>143226138</v>
       </c>
@@ -41304,7 +41304,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="386" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="386" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A386" s="291">
         <v>143220138</v>
       </c>
@@ -41324,7 +41324,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="387" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="387" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A387" s="291">
         <v>143140038</v>
       </c>
@@ -41344,7 +41344,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="388" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="388" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A388" s="290">
         <v>143510038</v>
       </c>
@@ -41358,7 +41358,7 @@
       <c r="E388" s="179"/>
       <c r="F388" s="282"/>
     </row>
-    <row r="389" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="389" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A389" s="313">
         <v>143180038</v>
       </c>
@@ -41378,7 +41378,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="390" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="390" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A390" s="291">
         <v>143630038</v>
       </c>
@@ -41398,7 +41398,7 @@
         <v>24990</v>
       </c>
     </row>
-    <row r="391" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="391" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A391" s="291">
         <v>143600038</v>
       </c>
@@ -41412,7 +41412,7 @@
       <c r="E391" s="114"/>
       <c r="F391" s="282"/>
     </row>
-    <row r="392" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="392" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A392" s="291">
         <v>143650038</v>
       </c>
@@ -41435,7 +41435,7 @@
         <v>3902</v>
       </c>
     </row>
-    <row r="393" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="393" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A393" s="290">
         <v>143470038</v>
       </c>
@@ -41449,7 +41449,7 @@
       <c r="E393" s="179"/>
       <c r="F393" s="282"/>
     </row>
-    <row r="394" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="394" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A394" s="290">
         <v>143370038</v>
       </c>
@@ -41469,7 +41469,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="395" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="395" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A395" s="290">
         <v>143390038</v>
       </c>
@@ -41492,7 +41492,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="396" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="396" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A396" s="290">
         <v>143130038</v>
       </c>
@@ -41515,7 +41515,7 @@
         <v>2144</v>
       </c>
     </row>
-    <row r="397" spans="1:7" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="397" spans="1:7" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A397" s="355">
         <v>143250038</v>
       </c>
@@ -41535,7 +41535,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="398" spans="1:7" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="398" spans="1:7" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A398" s="355">
         <v>143250138</v>
       </c>
@@ -41555,7 +41555,7 @@
         <v>25900</v>
       </c>
     </row>
-    <row r="399" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="399" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A399" s="290">
         <v>143410038</v>
       </c>
@@ -41575,7 +41575,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="400" spans="1:7" ht="13.8" ns3:dyDescent="0.25">
+    <row r="400" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A400" s="290">
         <v>143330038</v>
       </c>
@@ -41596,7 +41596,7 @@
       </c>
       <c r="G400" s="185"/>
     </row>
-    <row r="401" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="401" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A401" s="290">
         <v>143190038</v>
       </c>
@@ -41616,7 +41616,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="402" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="402" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A402" s="312">
         <v>143230038</v>
       </c>
@@ -41636,7 +41636,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="403" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="403" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A403" s="312">
         <v>143230138</v>
       </c>
@@ -41656,7 +41656,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="404" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="404" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A404" s="312">
         <v>143090038</v>
       </c>
@@ -41682,7 +41682,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="405" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="405" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A405" s="292">
         <v>143030038</v>
       </c>
@@ -41708,7 +41708,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="406" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="406" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A406" s="312">
         <v>143290038</v>
       </c>
@@ -41728,7 +41728,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="407" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="407" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A407" s="292">
         <v>143100038</v>
       </c>
@@ -41754,7 +41754,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="408" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="408" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A408" s="292">
         <v>143070038</v>
       </c>
@@ -41774,7 +41774,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="409" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="409" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A409" s="361">
         <v>143610438</v>
       </c>
@@ -41794,7 +41794,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="410" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="410" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A410" s="361">
         <v>143616738</v>
       </c>
@@ -41814,7 +41814,7 @@
         <v>27990</v>
       </c>
     </row>
-    <row r="411" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="411" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A411" s="361">
         <v>143610638</v>
       </c>
@@ -41834,7 +41834,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="412" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="412" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A412" s="361">
         <v>143610838</v>
       </c>
@@ -41854,7 +41854,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="413" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="413" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A413" s="361">
         <v>143611638</v>
       </c>
@@ -41874,7 +41874,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="414" spans="1:8" s="359" customFormat="1" ht="13.8" ns3:dyDescent="0.25">
+    <row r="414" spans="1:8" s="359" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A414" s="361">
         <v>143614838</v>
       </c>
@@ -41894,7 +41894,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="415" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="415" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A415" s="29">
         <v>143620438</v>
       </c>
@@ -41914,7 +41914,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="416" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="416" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A416" s="29">
         <v>143620638</v>
       </c>
@@ -41934,7 +41934,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="417" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="417" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A417" s="29">
         <v>143620838</v>
       </c>
@@ -41954,7 +41954,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="418" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="418" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A418" s="29">
         <v>143621638</v>
       </c>
@@ -41974,7 +41974,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="419" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="419" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A419" s="29">
         <v>143624838</v>
       </c>
@@ -41994,7 +41994,7 @@
         <v>25991</v>
       </c>
     </row>
-    <row r="420" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="420" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A420" s="29">
         <v>143660038</v>
       </c>
@@ -42014,7 +42014,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="421" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="421" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A421" s="29">
         <v>143660038</v>
       </c>
@@ -42034,7 +42034,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="422" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="422" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A422" s="29">
         <v>143660038</v>
       </c>
@@ -42054,7 +42054,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="423" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="423" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A423" s="29">
         <v>143660038</v>
       </c>
@@ -42074,7 +42074,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="424" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="424" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A424" s="29">
         <v>143660038</v>
       </c>
@@ -42094,7 +42094,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="425" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="425" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A425" s="47">
         <v>143700138</v>
       </c>
@@ -42114,7 +42114,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="426" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="426" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A426" s="47">
         <v>143700438</v>
       </c>
@@ -42134,7 +42134,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="427" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="427" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A427" s="47">
         <v>143700038</v>
       </c>
@@ -42154,7 +42154,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="428" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="428" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A428" s="47">
         <v>143700238</v>
       </c>
@@ -42174,7 +42174,7 @@
         <v>26990</v>
       </c>
     </row>
-    <row r="429" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="429" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A429" s="292">
         <v>143710038</v>
       </c>
@@ -42194,7 +42194,7 @@
         <v>25990</v>
       </c>
     </row>
-    <row r="430" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="430" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A430" s="292">
         <v>143770038</v>
       </c>
@@ -42220,7 +42220,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="431" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="431" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A431" s="292">
         <v>143790038</v>
       </c>
@@ -42246,7 +42246,7 @@
         <v>2173</v>
       </c>
     </row>
-    <row r="432" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="432" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A432" s="292">
         <v>143780038</v>
       </c>
@@ -42272,7 +42272,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="433" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="433" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A433" s="292">
         <v>143780138</v>
       </c>
@@ -42293,7 +42293,7 @@
       </c>
       <c r="G433" s="350"/>
     </row>
-    <row r="434" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="434" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A434" s="292">
         <v>143800038</v>
       </c>
@@ -42314,7 +42314,7 @@
       </c>
       <c r="G434" s="350"/>
     </row>
-    <row r="435" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="435" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A435" s="292">
         <v>143800138</v>
       </c>
@@ -42335,7 +42335,7 @@
       </c>
       <c r="G435" s="350"/>
     </row>
-    <row r="436" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="436" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A436" s="312">
         <v>143010038</v>
       </c>
@@ -42361,7 +42361,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="437" spans="1:8" ht="13.8" ns3:dyDescent="0.25">
+    <row r="437" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A437" s="314">
         <v>11111111</v>
       </c>
@@ -42373,7 +42373,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="438" spans="1:8" ns3:dyDescent="0.3">
+    <row r="438" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A438" s="292"/>
     </row>
     <row r="439">
@@ -51053,7 +51053,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="H218:K282">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H218:K282">
     <sortCondition ref="H218:H282"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -51123,8 +51123,8 @@
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.11811023622047245" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="11" orientation="portrait" ns4:id="rId1"/>
-  <drawing ns4:id="rId2"/>
+  <pageSetup scale="11" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: stock Cole 44 (13 disponibles), clienta Duhart en BD/web, tope por talla cole-43, flechas solo mobile, script stock BI, docs
- stock-data-catalogo-44.json: solo 13 modelos disponibles (definidos a mano)
- PLANILLA 43/44: clienta 16.388.334-1 en BASE DE DATOS OFICIAL fila 167, rango VLOOKUP a 400
- script-v2.js: overrides locales de cliente, tope por talla segun stock ERP, badge 'Quedan N', version plantillas
- catalogo-44: CLIENTES_LOCALES con pre-llenado; cole-43: flechas del modal solo en celular
- generate-stock-from-bi.ps1 (Cole 40-43, desactivado en auto_build.bat), SQL fix RPC clientes, CLAUDE.md

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PLANILLA 43 LISTA PRECIO FINAL.xlsx
+++ b/PLANILLA 43 LISTA PRECIO FINAL.xlsx
@@ -695,7 +695,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2389" uniqueCount="2389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2399" uniqueCount="2397">
   <si>
     <t>TRANSPORTE</t>
   </si>
@@ -8405,6 +8405,30 @@
   </si>
   <si>
     <t>BEIGE BOLSILLO RELOJERO 3  PINZAS</t>
+  </si>
+  <si>
+    <t>16.388.334-1</t>
+  </si>
+  <si>
+    <t>XIMENA ANDREA DUHART DUHART</t>
+  </si>
+  <si>
+    <t>LAGO LYNCH #45</t>
+  </si>
+  <si>
+    <t>costaneraporvenir@gmail.com</t>
+  </si>
+  <si>
+    <t>AL CONTADO</t>
+  </si>
+  <si>
+    <t>GRANDES TIENDAS DE VESTIR Y CALZADO</t>
+  </si>
+  <si>
+    <t>TIENDA ANTONELLA</t>
+  </si>
+  <si>
+    <t>REGION DE MAGALLANES - TIERRA DEL FUEGO</t>
   </si>
 </sst>
 </file>
@@ -23700,7 +23724,7 @@
       <c r="J1" s="437"/>
       <c r="K1" s="438"/>
       <c r="L1" s="396" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,3,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,3,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M1" s="397"/>
@@ -23727,7 +23751,7 @@
       <c r="J2" s="435"/>
       <c r="K2" s="386"/>
       <c r="L2" s="418" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,19,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,19,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M2" s="419"/>
@@ -23757,7 +23781,7 @@
       <c r="J3" s="435"/>
       <c r="K3" s="386"/>
       <c r="L3" s="418" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,5,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,5,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M3" s="419"/>
@@ -23784,7 +23808,7 @@
       <c r="J4" s="435"/>
       <c r="K4" s="386"/>
       <c r="L4" s="423" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,20,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,20,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M4" s="423"/>
@@ -23839,7 +23863,7 @@
       <c r="J6" s="406"/>
       <c r="K6" s="393"/>
       <c r="L6" s="426" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,21,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,21,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M6" s="427"/>
@@ -23851,7 +23875,7 @@
       </c>
       <c r="R6" s="393"/>
       <c r="S6" s="403" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,4,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,4,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="T6" s="400"/>
@@ -23864,7 +23888,7 @@
       </c>
       <c r="D7" s="298"/>
       <c r="E7" s="450" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,17,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,17,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="F7" s="450"/>
@@ -23876,7 +23900,7 @@
       <c r="J7" s="406"/>
       <c r="K7" s="393"/>
       <c r="L7" s="426" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,6,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,6,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M7" s="427"/>
@@ -23888,7 +23912,7 @@
       </c>
       <c r="R7" s="393"/>
       <c r="S7" s="403" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,18,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,18,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="T7" s="400"/>
@@ -23922,7 +23946,7 @@
       </c>
       <c r="R8" s="393"/>
       <c r="S8" s="399" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,9,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,9,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="T8" s="400"/>
@@ -23944,7 +23968,7 @@
       <c r="J9" s="408"/>
       <c r="K9" s="409"/>
       <c r="L9" s="441" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,7,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,7,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M9" s="442"/>
@@ -24007,7 +24031,7 @@
       <c r="J11" s="408"/>
       <c r="K11" s="409"/>
       <c r="L11" s="414" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,29,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,29,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M11" s="414"/>
@@ -24070,7 +24094,7 @@
       <c r="J13" s="404"/>
       <c r="K13" s="404"/>
       <c r="L13" s="405" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,24,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,24,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="M13" s="405"/>
@@ -24078,16 +24102,16 @@
       <c r="O13" s="405"/>
       <c r="P13" s="405"/>
       <c r="Q13" s="387" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,25,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,25,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="R13" s="387"/>
       <c r="S13" s="121" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,26,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,26,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
       <c r="T13" s="126" t="str">
-        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$166,28,0),"SIN INFORMACIÓN")</f>
+        <f>_xlfn.IFNA(VLOOKUP(L5,'BASE DE DATOS OFICIAL'!$A$4:$AC$400,28,0),"SIN INFORMACIÓN")</f>
         <v>SIN INFORMACIÓN</v>
       </c>
     </row>
@@ -76257,7 +76281,47 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="167" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="67" t="s">
+        <v>2389</v>
+      </c>
+      <c r="B167" s="67">
+        <v>163883341</v>
+      </c>
+      <c r="C167" s="61" t="s">
+        <v>2390</v>
+      </c>
+      <c r="D167" s="62" t="s">
+        <v>210</v>
+      </c>
+      <c r="E167" s="63" t="s">
+        <v>2391</v>
+      </c>
+      <c r="F167" s="62">
+        <v>950096525</v>
+      </c>
+      <c r="H167" s="67" t="s">
+        <v>2392</v>
+      </c>
+      <c r="Q167" s="62" t="s">
+        <v>2393</v>
+      </c>
+      <c r="R167" s="62">
+        <v>950096525</v>
+      </c>
+      <c r="S167" s="62" t="s">
+        <v>2394</v>
+      </c>
+      <c r="T167" s="62" t="s">
+        <v>2395</v>
+      </c>
+      <c r="U167" s="67" t="s">
+        <v>210</v>
+      </c>
+      <c r="V167" s="67" t="s">
+        <v>2396</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H65" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>

</xml_diff>